<commit_message>
release 0.3.1 chat polish and app lock
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="R817029fc39a24307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R9dfef767919f4505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="Rf80a014dad5a4d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R31d447d7da2c4ae1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -580,7 +580,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -627,8 +627,53 @@
         <x:fgColor rgb="FFFFF9E8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="5">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -651,11 +696,16 @@
         <x:color rgb="FFB8ACC7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFDED8E5"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -719,6 +769,103 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -729,7 +876,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D112" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="English text"/>
@@ -1893,6 +2040,402 @@
       </x:c>
       <x:c r="D80" s="28" t="str"/>
     </x:row>
+    <x:row r="81" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A81" s="36" t="str">
+        <x:v>typing_indicator</x:v>
+      </x:c>
+      <x:c r="B81" s="40" t="str">
+        <x:v>%1$s is typing</x:v>
+      </x:c>
+      <x:c r="C81" s="46" t="str">
+        <x:v>Chat typing indicator</x:v>
+      </x:c>
+      <x:c r="D81" s="46" t="str">
+        <x:v>%1$s = contact name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A82" s="36" t="str">
+        <x:v>image_attachment</x:v>
+      </x:c>
+      <x:c r="B82" s="40" t="str">
+        <x:v>%1$s image</x:v>
+      </x:c>
+      <x:c r="C82" s="46" t="str">
+        <x:v>Image attachment description</x:v>
+      </x:c>
+      <x:c r="D82" s="46" t="str">
+        <x:v>%1$s = file name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A83" s="36" t="str">
+        <x:v>file_attachment</x:v>
+      </x:c>
+      <x:c r="B83" s="40" t="str">
+        <x:v>%1$s file</x:v>
+      </x:c>
+      <x:c r="C83" s="46" t="str">
+        <x:v>File attachment description</x:v>
+      </x:c>
+      <x:c r="D83" s="46" t="str">
+        <x:v>%1$s = file name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A84" s="36" t="str">
+        <x:v>attachment_loading</x:v>
+      </x:c>
+      <x:c r="B84" s="40" t="str">
+        <x:v>Receiving original file…</x:v>
+      </x:c>
+      <x:c r="C84" s="46" t="str">
+        <x:v>Attachment preview progress</x:v>
+      </x:c>
+      <x:c r="D84" s="46"/>
+    </x:row>
+    <x:row r="85" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A85" s="36" t="str">
+        <x:v>attachment_unavailable</x:v>
+      </x:c>
+      <x:c r="B85" s="40" t="str">
+        <x:v>Original file is available when the sender is online.</x:v>
+      </x:c>
+      <x:c r="C85" s="46" t="str">
+        <x:v>Attachment preview fallback</x:v>
+      </x:c>
+      <x:c r="D85" s="46"/>
+    </x:row>
+    <x:row r="86" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A86" s="36" t="str">
+        <x:v>message_from_you</x:v>
+      </x:c>
+      <x:c r="B86" s="40" t="str">
+        <x:v>You</x:v>
+      </x:c>
+      <x:c r="C86" s="46" t="str">
+        <x:v>Message accessibility label</x:v>
+      </x:c>
+      <x:c r="D86" s="46"/>
+    </x:row>
+    <x:row r="87" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A87" s="36" t="str">
+        <x:v>message_from_contact</x:v>
+      </x:c>
+      <x:c r="B87" s="40" t="str">
+        <x:v>%1$s</x:v>
+      </x:c>
+      <x:c r="C87" s="46" t="str">
+        <x:v>Message accessibility label</x:v>
+      </x:c>
+      <x:c r="D87" s="46" t="str">
+        <x:v>%1$s = contact name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A88" s="36" t="str">
+        <x:v>message_accessibility</x:v>
+      </x:c>
+      <x:c r="B88" s="40" t="str">
+        <x:v>%1$s. %2$s. %3$s. %4$s</x:v>
+      </x:c>
+      <x:c r="C88" s="46" t="str">
+        <x:v>Message accessibility summary</x:v>
+      </x:c>
+      <x:c r="D88" s="46" t="str">
+        <x:v>%1$s = sender; %2$s = content; %3$s = time; %4$s = status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A89" s="36" t="str">
+        <x:v>receipt_status_read</x:v>
+      </x:c>
+      <x:c r="B89" s="40" t="str">
+        <x:v>Read</x:v>
+      </x:c>
+      <x:c r="C89" s="46" t="str">
+        <x:v>Read receipt accessibility label</x:v>
+      </x:c>
+      <x:c r="D89" s="46"/>
+    </x:row>
+    <x:row r="90" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A90" s="36" t="str">
+        <x:v>receipt_status_delivered</x:v>
+      </x:c>
+      <x:c r="B90" s="40" t="str">
+        <x:v>Delivered</x:v>
+      </x:c>
+      <x:c r="C90" s="46" t="str">
+        <x:v>Read receipt accessibility label</x:v>
+      </x:c>
+      <x:c r="D90" s="46"/>
+    </x:row>
+    <x:row r="91" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A91" s="36" t="str">
+        <x:v>receipt_status_sent</x:v>
+      </x:c>
+      <x:c r="B91" s="40" t="str">
+        <x:v>Sent</x:v>
+      </x:c>
+      <x:c r="C91" s="46" t="str">
+        <x:v>Read receipt accessibility label</x:v>
+      </x:c>
+      <x:c r="D91" s="46"/>
+    </x:row>
+    <x:row r="92" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A92" s="36" t="str">
+        <x:v>receipt_status_waiting</x:v>
+      </x:c>
+      <x:c r="B92" s="40" t="str">
+        <x:v>Waiting to send</x:v>
+      </x:c>
+      <x:c r="C92" s="46" t="str">
+        <x:v>Read receipt accessibility label</x:v>
+      </x:c>
+      <x:c r="D92" s="46"/>
+    </x:row>
+    <x:row r="93" ht="14.25" hidden="0" customHeight="1">
+      <x:c r="A93" s="37" t="str">
+        <x:v>attachment_transfer_failed</x:v>
+      </x:c>
+      <x:c r="B93" s="41" t="str">
+        <x:v>The original file could not be received.</x:v>
+      </x:c>
+      <x:c r="C93" s="47" t="str">
+        <x:v>Attachment transfer error</x:v>
+      </x:c>
+      <x:c r="D93" s="47"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="68" t="str">
+        <x:v>debug_key</x:v>
+      </x:c>
+      <x:c r="B94" s="71" t="str">
+        <x:v>Debug key</x:v>
+      </x:c>
+      <x:c r="C94" s="74" t="str">
+        <x:v>App lock and Settings label</x:v>
+      </x:c>
+      <x:c r="D94" s="74" t="str"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="69" t="str">
+        <x:v>debug_key_mask</x:v>
+      </x:c>
+      <x:c r="B95" s="72" t="str">
+        <x:v>**************</x:v>
+      </x:c>
+      <x:c r="C95" s="75" t="str">
+        <x:v>Masked debug key value in Settings</x:v>
+      </x:c>
+      <x:c r="D95" s="75" t="str">
+        <x:v>Always displays 14 asterisks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="69" t="str">
+        <x:v>debug_key_required</x:v>
+      </x:c>
+      <x:c r="B96" s="72" t="str">
+        <x:v>Debug key required</x:v>
+      </x:c>
+      <x:c r="C96" s="76" t="str">
+        <x:v>App unlock dialog title</x:v>
+      </x:c>
+      <x:c r="D96" s="76" t="str"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="69" t="str">
+        <x:v>debug_key_prompt</x:v>
+      </x:c>
+      <x:c r="B97" s="72" t="str">
+        <x:v>Need debug key, ask your developer for a key</x:v>
+      </x:c>
+      <x:c r="C97" s="75" t="str">
+        <x:v>App unlock dialog body</x:v>
+      </x:c>
+      <x:c r="D97" s="75" t="str"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="69" t="str">
+        <x:v>debug_key_incorrect</x:v>
+      </x:c>
+      <x:c r="B98" s="72" t="str">
+        <x:v>That debug key is incorrect.</x:v>
+      </x:c>
+      <x:c r="C98" s="76" t="str">
+        <x:v>App unlock validation</x:v>
+      </x:c>
+      <x:c r="D98" s="76" t="str"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="69" t="str">
+        <x:v>unlock</x:v>
+      </x:c>
+      <x:c r="B99" s="72" t="str">
+        <x:v>Unlock</x:v>
+      </x:c>
+      <x:c r="C99" s="75" t="str">
+        <x:v>App unlock action</x:v>
+      </x:c>
+      <x:c r="D99" s="75" t="str"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="69" t="str">
+        <x:v>create_debug_key</x:v>
+      </x:c>
+      <x:c r="B100" s="72" t="str">
+        <x:v>Create debug key</x:v>
+      </x:c>
+      <x:c r="C100" s="76" t="str">
+        <x:v>First-run app lock title</x:v>
+      </x:c>
+      <x:c r="D100" s="76" t="str"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="69" t="str">
+        <x:v>debug_key_first_setup_body</x:v>
+      </x:c>
+      <x:c r="B101" s="72" t="str">
+        <x:v>Need debug key, ask your developer for a key. Create a four-digit key for this phone.</x:v>
+      </x:c>
+      <x:c r="C101" s="75" t="str">
+        <x:v>First-run app lock body</x:v>
+      </x:c>
+      <x:c r="D101" s="75" t="str"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="69" t="str">
+        <x:v>save_debug_key</x:v>
+      </x:c>
+      <x:c r="B102" s="72" t="str">
+        <x:v>Save debug key</x:v>
+      </x:c>
+      <x:c r="C102" s="76" t="str">
+        <x:v>First-run app lock action</x:v>
+      </x:c>
+      <x:c r="D102" s="76" t="str"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="69" t="str">
+        <x:v>new_debug_key</x:v>
+      </x:c>
+      <x:c r="B103" s="72" t="str">
+        <x:v>New debug key</x:v>
+      </x:c>
+      <x:c r="C103" s="75" t="str">
+        <x:v>Debug key input label</x:v>
+      </x:c>
+      <x:c r="D103" s="75" t="str"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="69" t="str">
+        <x:v>confirm_debug_key</x:v>
+      </x:c>
+      <x:c r="B104" s="72" t="str">
+        <x:v>Confirm debug key</x:v>
+      </x:c>
+      <x:c r="C104" s="76" t="str">
+        <x:v>Debug key confirmation label</x:v>
+      </x:c>
+      <x:c r="D104" s="76" t="str"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="69" t="str">
+        <x:v>debug_key_four_digits_error</x:v>
+      </x:c>
+      <x:c r="B105" s="72" t="str">
+        <x:v>Enter exactly four digits in both fields.</x:v>
+      </x:c>
+      <x:c r="C105" s="75" t="str">
+        <x:v>Debug key validation</x:v>
+      </x:c>
+      <x:c r="D105" s="75" t="str"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="69" t="str">
+        <x:v>debug_key_mismatch_error</x:v>
+      </x:c>
+      <x:c r="B106" s="72" t="str">
+        <x:v>The debug keys do not match.</x:v>
+      </x:c>
+      <x:c r="C106" s="76" t="str">
+        <x:v>Debug key validation</x:v>
+      </x:c>
+      <x:c r="D106" s="76" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="69" t="str">
+        <x:v>debug_key_save_error</x:v>
+      </x:c>
+      <x:c r="B107" s="72" t="str">
+        <x:v>The debug key could not be saved.</x:v>
+      </x:c>
+      <x:c r="C107" s="75" t="str">
+        <x:v>Debug key persistence error</x:v>
+      </x:c>
+      <x:c r="D107" s="75" t="str"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="69" t="str">
+        <x:v>debug_key_accessibility</x:v>
+      </x:c>
+      <x:c r="B108" s="72" t="str">
+        <x:v>Debug key. Hidden value. Tap seven times within three seconds to reset it.</x:v>
+      </x:c>
+      <x:c r="C108" s="76" t="str">
+        <x:v>Settings accessibility label</x:v>
+      </x:c>
+      <x:c r="D108" s="76" t="str"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="69" t="str">
+        <x:v>reset_debug_key</x:v>
+      </x:c>
+      <x:c r="B109" s="72" t="str">
+        <x:v>Reset debug key</x:v>
+      </x:c>
+      <x:c r="C109" s="75" t="str">
+        <x:v>Settings debug key dialog title and action</x:v>
+      </x:c>
+      <x:c r="D109" s="75" t="str"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="69" t="str">
+        <x:v>reset_debug_key_body</x:v>
+      </x:c>
+      <x:c r="B110" s="72" t="str">
+        <x:v>Create and confirm a new four-digit debug key.</x:v>
+      </x:c>
+      <x:c r="C110" s="76" t="str">
+        <x:v>Settings debug key dialog body</x:v>
+      </x:c>
+      <x:c r="D110" s="76" t="str"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="69" t="str">
+        <x:v>debug_key_updated</x:v>
+      </x:c>
+      <x:c r="B111" s="72" t="str">
+        <x:v>Debug key updated.</x:v>
+      </x:c>
+      <x:c r="C111" s="75" t="str">
+        <x:v>Settings debug key result</x:v>
+      </x:c>
+      <x:c r="D111" s="75" t="str"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="70" t="str">
+        <x:v>cancel</x:v>
+      </x:c>
+      <x:c r="B112" s="73" t="str">
+        <x:v>Cancel</x:v>
+      </x:c>
+      <x:c r="C112" s="77" t="str">
+        <x:v>Dialog action</x:v>
+      </x:c>
+      <x:c r="D112" s="77" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -1900,7 +2443,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77759dacdc344cbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2a624aee674786"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
release 0.3.2 expressive chat and keypad lock
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="Rf80a014dad5a4d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R31d447d7da2c4ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="Rece746c68c6f4d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R8d488e51a468429b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -580,7 +580,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -672,6 +672,16 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -705,7 +715,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="78">
+  <x:cellXfs count="93">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -868,6 +878,27 @@
     <x:xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -876,7 +907,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D112" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="English text"/>
@@ -2436,6 +2467,286 @@
       </x:c>
       <x:c r="D112" s="77" t="str"/>
     </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>open_emoji_picker</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Open emoji picker</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Chat composer accessibility label</x:v>
+      </x:c>
+      <x:c r="D113"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>close_emoji_picker</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>Close emoji picker</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>Chat composer accessibility label</x:v>
+      </x:c>
+      <x:c r="D114"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>insert_emoji</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>Insert emoji %1$s</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>Emoji button accessibility label</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>%1$s = emoji</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>link_preview_accessibility</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>Link preview for %1$s: %2$s</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>Link preview accessibility summary</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>%1$s = site; %2$s = page title</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>open_link</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>Open link</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>Link preview action label</x:v>
+      </x:c>
+      <x:c r="D117"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="84" t="str">
+        <x:v>switch_to_light_theme</x:v>
+      </x:c>
+      <x:c r="B118" s="90" t="str">
+        <x:v>Switch to light theme</x:v>
+      </x:c>
+      <x:c r="C118" s="66" t="str">
+        <x:v>Chat header theme toggle</x:v>
+      </x:c>
+      <x:c r="D118" s="66" t="str"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="85" t="str">
+        <x:v>switch_to_dark_theme</x:v>
+      </x:c>
+      <x:c r="B119" s="91" t="str">
+        <x:v>Switch to dark theme</x:v>
+      </x:c>
+      <x:c r="C119" s="67" t="str">
+        <x:v>Chat header theme toggle</x:v>
+      </x:c>
+      <x:c r="D119" s="67" t="str"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="85" t="str">
+        <x:v>appearance</x:v>
+      </x:c>
+      <x:c r="B120" s="91" t="str">
+        <x:v>Appearance</x:v>
+      </x:c>
+      <x:c r="C120" s="67" t="str">
+        <x:v>Settings section</x:v>
+      </x:c>
+      <x:c r="D120" s="67" t="str"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="85" t="str">
+        <x:v>theme_system</x:v>
+      </x:c>
+      <x:c r="B121" s="91" t="str">
+        <x:v>Follow system</x:v>
+      </x:c>
+      <x:c r="C121" s="67" t="str">
+        <x:v>Theme preference</x:v>
+      </x:c>
+      <x:c r="D121" s="67" t="str"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="85" t="str">
+        <x:v>theme_light</x:v>
+      </x:c>
+      <x:c r="B122" s="91" t="str">
+        <x:v>Light</x:v>
+      </x:c>
+      <x:c r="C122" s="67" t="str">
+        <x:v>Theme preference</x:v>
+      </x:c>
+      <x:c r="D122" s="67" t="str"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="85" t="str">
+        <x:v>theme_dark</x:v>
+      </x:c>
+      <x:c r="B123" s="91" t="str">
+        <x:v>Dark</x:v>
+      </x:c>
+      <x:c r="C123" s="67" t="str">
+        <x:v>Theme preference</x:v>
+      </x:c>
+      <x:c r="D123" s="67" t="str"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="85" t="str">
+        <x:v>send_message_hint</x:v>
+      </x:c>
+      <x:c r="B124" s="91" t="str">
+        <x:v>Send message. Touch and hold to adjust message emphasis.</x:v>
+      </x:c>
+      <x:c r="C124" s="67" t="str">
+        <x:v>Send button accessibility hint</x:v>
+      </x:c>
+      <x:c r="D124" s="67" t="str"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="85" t="str">
+        <x:v>message_emphasis_preview</x:v>
+      </x:c>
+      <x:c r="B125" s="91" t="str">
+        <x:v>Message emphasis preview</x:v>
+      </x:c>
+      <x:c r="C125" s="67" t="str">
+        <x:v>Hold-to-send preview accessibility</x:v>
+      </x:c>
+      <x:c r="D125" s="67" t="str"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="85" t="str">
+        <x:v>emphasis_normal</x:v>
+      </x:c>
+      <x:c r="B126" s="91" t="str">
+        <x:v>Normal size</x:v>
+      </x:c>
+      <x:c r="C126" s="67" t="str">
+        <x:v>Message emphasis accessibility</x:v>
+      </x:c>
+      <x:c r="D126" s="67" t="str"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="85" t="str">
+        <x:v>emphasis_low</x:v>
+      </x:c>
+      <x:c r="B127" s="91" t="str">
+        <x:v>Low emphasis</x:v>
+      </x:c>
+      <x:c r="C127" s="67" t="str">
+        <x:v>Message emphasis accessibility</x:v>
+      </x:c>
+      <x:c r="D127" s="67" t="str"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="85" t="str">
+        <x:v>emphasis_medium</x:v>
+      </x:c>
+      <x:c r="B128" s="91" t="str">
+        <x:v>Medium emphasis</x:v>
+      </x:c>
+      <x:c r="C128" s="67" t="str">
+        <x:v>Message emphasis accessibility</x:v>
+      </x:c>
+      <x:c r="D128" s="67" t="str"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="85" t="str">
+        <x:v>emphasis_high</x:v>
+      </x:c>
+      <x:c r="B129" s="91" t="str">
+        <x:v>High emphasis</x:v>
+      </x:c>
+      <x:c r="C129" s="67" t="str">
+        <x:v>Message emphasis accessibility</x:v>
+      </x:c>
+      <x:c r="D129" s="67" t="str"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="85" t="str">
+        <x:v>emphasis_maximum</x:v>
+      </x:c>
+      <x:c r="B130" s="91" t="str">
+        <x:v>Maximum emphasis</x:v>
+      </x:c>
+      <x:c r="C130" s="67" t="str">
+        <x:v>Message emphasis accessibility</x:v>
+      </x:c>
+      <x:c r="D130" s="67" t="str"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="85" t="str">
+        <x:v>send_cancelled</x:v>
+      </x:c>
+      <x:c r="B131" s="91" t="str">
+        <x:v>Send cancelled</x:v>
+      </x:c>
+      <x:c r="C131" s="67" t="str">
+        <x:v>Send gesture accessibility announcement</x:v>
+      </x:c>
+      <x:c r="D131" s="67" t="str"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="85" t="str">
+        <x:v>drag_left_to_reduce</x:v>
+      </x:c>
+      <x:c r="B132" s="91" t="str">
+        <x:v>Drag left to reduce · move up to cancel</x:v>
+      </x:c>
+      <x:c r="C132" s="67" t="str">
+        <x:v>Hold-to-send gesture instruction</x:v>
+      </x:c>
+      <x:c r="D132" s="67" t="str"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="85" t="str">
+        <x:v>open_source_licenses</x:v>
+      </x:c>
+      <x:c r="B133" s="91" t="str">
+        <x:v>Open-source licenses</x:v>
+      </x:c>
+      <x:c r="C133" s="67" t="str">
+        <x:v>Settings action</x:v>
+      </x:c>
+      <x:c r="D133" s="67" t="str"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="85" t="str">
+        <x:v>google_sans_flex_license_title</x:v>
+      </x:c>
+      <x:c r="B134" s="91" t="str">
+        <x:v>Google Sans Flex license</x:v>
+      </x:c>
+      <x:c r="C134" s="67" t="str">
+        <x:v>Font license dialog title</x:v>
+      </x:c>
+      <x:c r="D134" s="67" t="str"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="86" t="str">
+        <x:v>close</x:v>
+      </x:c>
+      <x:c r="B135" s="92" t="str">
+        <x:v>Close</x:v>
+      </x:c>
+      <x:c r="C135" s="22" t="str">
+        <x:v>Dialog action</x:v>
+      </x:c>
+      <x:c r="D135" s="22" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -2443,7 +2754,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2a624aee674786"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b3c481b1aef4e5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update Android chat app
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="Rece746c68c6f4d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R8d488e51a468429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="R74736fa91105427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R2763911c1983436e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,15 +74,9 @@
     <x:t xml:space="preserve">status_relay_offline</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Relay offline</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">status_connecting_relay</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Connecting to relay</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">settings</x:t>
   </x:si>
   <x:si>
@@ -131,22 +125,13 @@
     <x:t xml:space="preserve">pairing_card_registered_body</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Code active on the relay. Enter it on the private web page from any location.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">retry_relay_connection</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Retry relay connection</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pairing error action</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">pairing_registering</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Registering this code with the relay…</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pairing progress</x:t>
@@ -540,7 +525,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -579,8 +564,13 @@
       <x:color rgb="FF5F4500"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -682,6 +672,26 @@
         <x:fgColor rgb="FFFFF9E8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F3FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -715,7 +725,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="93">
+  <x:cellXfs count="113">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -899,6 +909,46 @@
     <x:xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -907,7 +957,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidStringsTable" displayName="AndroidStringsTable" ref="A4:D123" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Key"/>
     <x:tableColumn id="2" name="English text"/>
@@ -1213,8 +1263,8 @@
       <x:c r="A10" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>21</x:v>
+      <x:c r="B10" s="3" t="str">
+        <x:v>Offline</x:v>
       </x:c>
       <x:c r="C10" s="4" t="s">
         <x:v>17</x:v>
@@ -1223,10 +1273,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>Connecting</x:v>
       </x:c>
       <x:c r="C11" s="4" t="s">
         <x:v>17</x:v>
@@ -1235,629 +1285,629 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C12" s="4" t="s">
-        <x:v>26</x:v>
       </x:c>
       <x:c r="D12" s="4"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="s">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C13" s="4" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="D13" s="4"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="C14" s="4" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="D14" s="4"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C15" s="4" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="D15" s="4"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="C16" s="4" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="D16" s="4"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B17" s="3" t="s">
-        <x:v>40</x:v>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B17" s="3" t="str">
+        <x:v>Code active. Enter it on the private web page from any location.</x:v>
       </x:c>
       <x:c r="C17" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D17" s="4"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="s">
-        <x:v>42</x:v>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B18" s="3" t="str">
+        <x:v>Retry connection</x:v>
       </x:c>
       <x:c r="C18" s="4" t="s">
-        <x:v>43</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D18" s="4"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="s">
-        <x:v>45</x:v>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="str">
+        <x:v>Registering this code…</x:v>
       </x:c>
       <x:c r="C19" s="4" t="s">
-        <x:v>46</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D19" s="4"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="s">
-        <x:v>47</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
-        <x:v>48</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C20" s="4" t="s">
-        <x:v>49</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D20" s="4"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
-        <x:v>51</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C21" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D21" s="4"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
-        <x:v>54</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C22" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D22" s="4"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
-        <x:v>56</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C23" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D23" s="4"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C24" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D24" s="4"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C25" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D25" s="4"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="2" t="s">
-        <x:v>61</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C26" s="4" t="s">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D26" s="4"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2" t="s">
-        <x:v>63</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C27" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D27" s="4"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2" t="s">
-        <x:v>66</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C28" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D28" s="4"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
-        <x:v>69</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C29" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D29" s="4"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
-        <x:v>71</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C30" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D30" s="4"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="2" t="s">
-        <x:v>72</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C31" s="4" t="s">
-        <x:v>74</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D31" s="4"/>
     </x:row>
     <x:row r="32" ht="28.5">
       <x:c r="A32" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
-        <x:v>76</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C32" s="4" t="s">
-        <x:v>77</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D32" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C33" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D33" s="4"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
-        <x:v>83</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C34" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D34" s="4"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
-        <x:v>85</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C35" s="4" t="s">
-        <x:v>86</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D35" s="4"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
-        <x:v>88</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C36" s="4" t="s">
-        <x:v>89</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D36" s="4"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="2" t="s">
-        <x:v>90</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
-        <x:v>91</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C37" s="4" t="s">
-        <x:v>92</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D37" s="4"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
-        <x:v>94</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C38" s="4" t="s">
-        <x:v>95</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D38" s="4"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="2" t="s">
-        <x:v>96</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C39" s="4" t="s">
-        <x:v>95</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D39" s="4"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="2" t="s">
-        <x:v>98</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B40" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C40" s="4" t="s">
-        <x:v>100</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D40" s="4"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2" t="s">
-        <x:v>101</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B41" s="3" t="s">
-        <x:v>102</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C41" s="4" t="s">
-        <x:v>103</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D41" s="4"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B42" s="3" t="s">
-        <x:v>105</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C42" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D42" s="4"/>
     </x:row>
     <x:row r="43" ht="28.5">
       <x:c r="A43" s="2" t="s">
-        <x:v>107</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B43" s="3" t="s">
-        <x:v>108</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C43" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D43" s="4"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2" t="s">
-        <x:v>109</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B44" s="3" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C44" s="4" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D44" s="4"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B45" s="3" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C45" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D45" s="4"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="2" t="s">
-        <x:v>115</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B46" s="3" t="s">
-        <x:v>116</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C46" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D46" s="4"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="s">
-        <x:v>117</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B47" s="3" t="s">
-        <x:v>118</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C47" s="4" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D47" s="4"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B48" s="3" t="s">
-        <x:v>120</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C48" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D48" s="4"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="s">
-        <x:v>121</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B49" s="3" t="s">
-        <x:v>122</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C49" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D49" s="4"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B50" s="3" t="s">
-        <x:v>124</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C50" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D50" s="4"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B51" s="3" t="s">
-        <x:v>127</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C51" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D51" s="4"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="2" t="s">
-        <x:v>128</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B52" s="3" t="s">
-        <x:v>129</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="C52" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D52" s="4"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2" t="s">
-        <x:v>131</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B53" s="3" t="s">
-        <x:v>132</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C53" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D53" s="4"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2" t="s">
-        <x:v>133</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B54" s="3" t="s">
-        <x:v>134</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C54" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D54" s="4"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="2" t="s">
-        <x:v>135</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B55" s="3" t="s">
-        <x:v>136</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C55" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D55" s="4"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="2" t="s">
-        <x:v>137</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B56" s="3" t="s">
-        <x:v>138</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="C56" s="4" t="s">
-        <x:v>139</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D56" s="4"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="2" t="s">
-        <x:v>140</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B57" s="3" t="s">
-        <x:v>141</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C57" s="4" t="s">
-        <x:v>142</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="D57" s="4"/>
     </x:row>
     <x:row r="58" ht="28.5">
       <x:c r="A58" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B58" s="3" t="s">
-        <x:v>144</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C58" s="4" t="s">
-        <x:v>145</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="D58" s="4"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="2" t="s">
-        <x:v>146</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B59" s="3" t="s">
-        <x:v>147</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="C59" s="4" t="s">
-        <x:v>148</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D59" s="4"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="2" t="s">
-        <x:v>149</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B60" s="3" t="s">
-        <x:v>150</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C60" s="4" t="s">
-        <x:v>151</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D60" s="4"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="2" t="s">
-        <x:v>152</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B61" s="3" t="s">
-        <x:v>153</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="C61" s="4" t="s">
-        <x:v>154</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="D61" s="4"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2" t="s">
-        <x:v>155</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B62" s="3" t="s">
-        <x:v>156</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C62" s="4" t="s">
-        <x:v>157</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D62" s="4" t="s">
-        <x:v>158</x:v>
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B63" s="6" t="s">
-        <x:v>160</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>161</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D63" s="7"/>
     </x:row>
@@ -2533,63 +2583,73 @@
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="84" t="str">
-        <x:v>switch_to_light_theme</x:v>
+        <x:v>message_sent_at</x:v>
       </x:c>
       <x:c r="B118" s="90" t="str">
-        <x:v>Switch to light theme</x:v>
+        <x:v>Sent %1$s</x:v>
       </x:c>
       <x:c r="C118" s="66" t="str">
-        <x:v>Chat header theme toggle</x:v>
-      </x:c>
-      <x:c r="D118" s="66" t="str"/>
+        <x:v>Read receipt disclosure</x:v>
+      </x:c>
+      <x:c r="D118" s="66" t="str">
+        <x:v>%1$s = sent time</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="85" t="str">
-        <x:v>switch_to_dark_theme</x:v>
+        <x:v>message_read_at</x:v>
       </x:c>
       <x:c r="B119" s="91" t="str">
-        <x:v>Switch to dark theme</x:v>
+        <x:v>Read %1$s</x:v>
       </x:c>
       <x:c r="C119" s="67" t="str">
-        <x:v>Chat header theme toggle</x:v>
-      </x:c>
-      <x:c r="D119" s="67" t="str"/>
+        <x:v>Read receipt disclosure</x:v>
+      </x:c>
+      <x:c r="D119" s="67" t="str">
+        <x:v>%1$s = read time</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="85" t="str">
-        <x:v>appearance</x:v>
+        <x:v>photo_count</x:v>
       </x:c>
       <x:c r="B120" s="91" t="str">
-        <x:v>Appearance</x:v>
+        <x:v>%1$d photos</x:v>
       </x:c>
       <x:c r="C120" s="67" t="str">
-        <x:v>Settings section</x:v>
-      </x:c>
-      <x:c r="D120" s="67" t="str"/>
+        <x:v>Multiple-image message summary</x:v>
+      </x:c>
+      <x:c r="D120" s="67" t="str">
+        <x:v>%1$d = image count</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="85" t="str">
-        <x:v>theme_system</x:v>
+        <x:v>attachment_count</x:v>
       </x:c>
       <x:c r="B121" s="91" t="str">
-        <x:v>Follow system</x:v>
+        <x:v>%1$d attachments</x:v>
       </x:c>
       <x:c r="C121" s="67" t="str">
-        <x:v>Theme preference</x:v>
-      </x:c>
-      <x:c r="D121" s="67" t="str"/>
+        <x:v>Multiple-attachment message summary</x:v>
+      </x:c>
+      <x:c r="D121" s="67" t="str">
+        <x:v>%1$d = attachment count</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="85" t="str">
-        <x:v>theme_light</x:v>
+        <x:v>image_position</x:v>
       </x:c>
       <x:c r="B122" s="91" t="str">
-        <x:v>Light</x:v>
+        <x:v>Image %1$d of %2$d</x:v>
       </x:c>
       <x:c r="C122" s="67" t="str">
-        <x:v>Theme preference</x:v>
-      </x:c>
-      <x:c r="D122" s="67" t="str"/>
+        <x:v>Carousel image accessibility label</x:v>
+      </x:c>
+      <x:c r="D122" s="67" t="str">
+        <x:v>%1$d = image position; %2$d = image count</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="85" t="str">
@@ -2601,7 +2661,7 @@
       <x:c r="C123" s="67" t="str">
         <x:v>Theme preference</x:v>
       </x:c>
-      <x:c r="D123" s="67" t="str"/>
+      <x:c r="D123" s="67"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="85" t="str">
@@ -2746,6 +2806,284 @@
         <x:v>Dialog action</x:v>
       </x:c>
       <x:c r="D135" s="22" t="str"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="109" t="str">
+        <x:v>selected_count</x:v>
+      </x:c>
+      <x:c r="B136" s="111" t="str">
+        <x:v>%1$d selected</x:v>
+      </x:c>
+      <x:c r="C136" s="22" t="str">
+        <x:v>Chat selection header</x:v>
+      </x:c>
+      <x:c r="D136" s="22" t="str">
+        <x:v>%1$d = selected message count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="110" t="str">
+        <x:v>clear_selection</x:v>
+      </x:c>
+      <x:c r="B137" s="112" t="str">
+        <x:v>Clear selection</x:v>
+      </x:c>
+      <x:c r="C137" s="25" t="str">
+        <x:v>Chat selection header action</x:v>
+      </x:c>
+      <x:c r="D137" s="25"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="110" t="str">
+        <x:v>reply</x:v>
+      </x:c>
+      <x:c r="B138" s="112" t="str">
+        <x:v>Reply</x:v>
+      </x:c>
+      <x:c r="C138" s="25" t="str">
+        <x:v>Message action</x:v>
+      </x:c>
+      <x:c r="D138" s="25"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="110" t="str">
+        <x:v>edit</x:v>
+      </x:c>
+      <x:c r="B139" s="112" t="str">
+        <x:v>Edit</x:v>
+      </x:c>
+      <x:c r="C139" s="25" t="str">
+        <x:v>Message action</x:v>
+      </x:c>
+      <x:c r="D139" s="25"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="110" t="str">
+        <x:v>delete</x:v>
+      </x:c>
+      <x:c r="B140" s="112" t="str">
+        <x:v>Delete</x:v>
+      </x:c>
+      <x:c r="C140" s="25" t="str">
+        <x:v>Message action</x:v>
+      </x:c>
+      <x:c r="D140" s="25"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="110" t="str">
+        <x:v>delete_message_title</x:v>
+      </x:c>
+      <x:c r="B141" s="112" t="str">
+        <x:v>Delete message?</x:v>
+      </x:c>
+      <x:c r="C141" s="25" t="str">
+        <x:v>Delete confirmation dialog</x:v>
+      </x:c>
+      <x:c r="D141" s="25"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="110" t="str">
+        <x:v>delete_for_me</x:v>
+      </x:c>
+      <x:c r="B142" s="112" t="str">
+        <x:v>Delete for me</x:v>
+      </x:c>
+      <x:c r="C142" s="25" t="str">
+        <x:v>Delete confirmation action</x:v>
+      </x:c>
+      <x:c r="D142" s="25"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="110" t="str">
+        <x:v>delete_for_both</x:v>
+      </x:c>
+      <x:c r="B143" s="112" t="str">
+        <x:v>Delete for both</x:v>
+      </x:c>
+      <x:c r="C143" s="25" t="str">
+        <x:v>Delete confirmation action</x:v>
+      </x:c>
+      <x:c r="D143" s="25"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="110" t="str">
+        <x:v>message_deleted</x:v>
+      </x:c>
+      <x:c r="B144" s="112" t="str">
+        <x:v>This message was deleted.</x:v>
+      </x:c>
+      <x:c r="C144" s="25" t="str">
+        <x:v>Deleted message placeholder</x:v>
+      </x:c>
+      <x:c r="D144" s="25"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="110" t="str">
+        <x:v>original_message_unavailable</x:v>
+      </x:c>
+      <x:c r="B145" s="112" t="str">
+        <x:v>Original message unavailable</x:v>
+      </x:c>
+      <x:c r="C145" s="25" t="str">
+        <x:v>Reply quote placeholder</x:v>
+      </x:c>
+      <x:c r="D145" s="25"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="110" t="str">
+        <x:v>original_message</x:v>
+      </x:c>
+      <x:c r="B146" s="112" t="str">
+        <x:v>Original message</x:v>
+      </x:c>
+      <x:c r="C146" s="25" t="str">
+        <x:v>Reply quote sender fallback</x:v>
+      </x:c>
+      <x:c r="D146" s="25"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="110" t="str">
+        <x:v>replying_to</x:v>
+      </x:c>
+      <x:c r="B147" s="112" t="str">
+        <x:v>Replying to</x:v>
+      </x:c>
+      <x:c r="C147" s="25" t="str">
+        <x:v>Composer reply state</x:v>
+      </x:c>
+      <x:c r="D147" s="25"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="110" t="str">
+        <x:v>editing_message</x:v>
+      </x:c>
+      <x:c r="B148" s="112" t="str">
+        <x:v>Editing message</x:v>
+      </x:c>
+      <x:c r="C148" s="25" t="str">
+        <x:v>Composer edit state</x:v>
+      </x:c>
+      <x:c r="D148" s="25"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="110" t="str">
+        <x:v>cancel_reply</x:v>
+      </x:c>
+      <x:c r="B149" s="112" t="str">
+        <x:v>Cancel reply</x:v>
+      </x:c>
+      <x:c r="C149" s="25" t="str">
+        <x:v>Composer reply action</x:v>
+      </x:c>
+      <x:c r="D149" s="25"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="110" t="str">
+        <x:v>cancel_edit</x:v>
+      </x:c>
+      <x:c r="B150" s="112" t="str">
+        <x:v>Cancel edit</x:v>
+      </x:c>
+      <x:c r="C150" s="25" t="str">
+        <x:v>Composer edit action</x:v>
+      </x:c>
+      <x:c r="D150" s="25"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="110" t="str">
+        <x:v>edited</x:v>
+      </x:c>
+      <x:c r="B151" s="112" t="str">
+        <x:v>edited</x:v>
+      </x:c>
+      <x:c r="C151" s="25" t="str">
+        <x:v>Edited message label</x:v>
+      </x:c>
+      <x:c r="D151" s="25"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="110" t="str">
+        <x:v>selected_message</x:v>
+      </x:c>
+      <x:c r="B152" s="112" t="str">
+        <x:v>Selected message</x:v>
+      </x:c>
+      <x:c r="C152" s="25" t="str">
+        <x:v>Selected message indicator</x:v>
+      </x:c>
+      <x:c r="D152" s="25"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>switch_to_light_theme</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>Switch to light theme</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>Chat header theme toggle</x:v>
+      </x:c>
+      <x:c r="D153"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>switch_to_dark_theme</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>Switch to dark theme</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>Chat header theme toggle</x:v>
+      </x:c>
+      <x:c r="D154"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>appearance</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>Appearance</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>Settings section</x:v>
+      </x:c>
+      <x:c r="D155"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>theme_system</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>Follow system</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>Theme preference</x:v>
+      </x:c>
+      <x:c r="D156"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>theme_light</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>Light</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>Theme preference</x:v>
+      </x:c>
+      <x:c r="D157"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>app_version</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>Settings information</x:v>
+      </x:c>
+      <x:c r="D158"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2754,7 +3092,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b3c481b1aef4e5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re30a1bb065a64801"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2769,56 +3107,56 @@
   <x:sheetData>
     <x:row r="1" ht="32.099998474121094" customHeight="1">
       <x:c r="A1" s="13" t="s">
-        <x:v>162</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B1" s="13"/>
     </x:row>
     <x:row r="3" ht="15">
       <x:c r="A3" s="8" t="s">
-        <x:v>163</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B3" s="9" t="s">
-        <x:v>164</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
       <x:c r="A4" s="8" t="s">
-        <x:v>165</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B4" s="9" t="s">
-        <x:v>166</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
       <x:c r="A5" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B5" s="9" t="s">
-        <x:v>168</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
       <x:c r="A6" s="8" t="s">
-        <x:v>169</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B6" s="9" t="s">
-        <x:v>170</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
       <x:c r="A7" s="8" t="s">
-        <x:v>171</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>172</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="10" t="s">
-        <x:v>173</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B9" s="10" t="s">
-        <x:v>174</x:v>
+        <x:v>169</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Support one web and one Android pairing claim
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="Ra62bdfb9a631414d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R1cf84f8c31f24796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="R9b077babf4ea4a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R5b8b03f69232452d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -269,31 +269,19 @@
     <x:t xml:space="preserve">web_pairing_code</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Web pairing code</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pairing screen heading</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">pairing_available_body</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Enter this code on the web portal to connect chat and storage to this phone.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pairing screen</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">pairing_claimed_body</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">This phone is already paired. Create a new code only to replace the paired browser.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">pairing_once_note</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A code works once. Rotate it only when pairing a replacement browser.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pairing screen note</x:t>
@@ -1619,325 +1607,325 @@
       <x:c r="A37" s="2" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B37" s="3" t="s">
+      <x:c r="B37" s="3" t="str">
+        <x:v>Pairing code</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="C37" s="4" t="s">
-        <x:v>87</x:v>
       </x:c>
       <x:c r="D37" s="4"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="2" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="str">
+        <x:v>Use this code once in a web browser and once on another Android phone.</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="B38" s="3" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="C38" s="4" t="s">
-        <x:v>90</x:v>
       </x:c>
       <x:c r="D38" s="4"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="2" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="B39" s="3" t="s">
-        <x:v>92</x:v>
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="str">
+        <x:v>This code has been used by both a web browser and an Android phone. Create a new code to pair replacements.</x:v>
       </x:c>
       <x:c r="C39" s="4" t="s">
-        <x:v>90</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D39" s="4"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="2" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="B40" s="3" t="s">
-        <x:v>94</x:v>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="str">
+        <x:v>Each code has one web slot and one Android slot. Existing paired devices stay connected after the code closes.</x:v>
       </x:c>
       <x:c r="C40" s="4" t="s">
-        <x:v>95</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D40" s="4"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2" t="s">
-        <x:v>96</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B41" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C41" s="4" t="s">
-        <x:v>98</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D41" s="4"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2" t="s">
-        <x:v>99</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B42" s="3" t="s">
-        <x:v>100</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C42" s="4" t="s">
-        <x:v>101</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D42" s="4"/>
     </x:row>
     <x:row r="43" ht="28.5">
       <x:c r="A43" s="2" t="s">
-        <x:v>102</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B43" s="3" t="s">
-        <x:v>103</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C43" s="4" t="s">
-        <x:v>101</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D43" s="4"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B44" s="3" t="s">
-        <x:v>105</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C44" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D44" s="4"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="2" t="s">
-        <x:v>107</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B45" s="3" t="s">
-        <x:v>108</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C45" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D45" s="4"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="2" t="s">
-        <x:v>110</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B46" s="3" t="s">
-        <x:v>111</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C46" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D46" s="4"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B47" s="3" t="s">
-        <x:v>113</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C47" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D47" s="4"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B48" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C48" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D48" s="4"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="s">
-        <x:v>116</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B49" s="3" t="s">
-        <x:v>117</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C49" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D49" s="4"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="2" t="s">
-        <x:v>118</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B50" s="3" t="s">
-        <x:v>119</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C50" s="4" t="s">
-        <x:v>120</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D50" s="4"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2" t="s">
-        <x:v>121</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B51" s="3" t="s">
-        <x:v>122</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="C51" s="4" t="s">
-        <x:v>120</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D51" s="4"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B52" s="3" t="s">
-        <x:v>124</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C52" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D52" s="4"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B53" s="3" t="s">
-        <x:v>127</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C53" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D53" s="4"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2" t="s">
-        <x:v>128</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B54" s="3" t="s">
-        <x:v>129</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="C54" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D54" s="4"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B55" s="3" t="s">
-        <x:v>131</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C55" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D55" s="4"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="2" t="s">
-        <x:v>132</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B56" s="3" t="s">
-        <x:v>133</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C56" s="4" t="s">
-        <x:v>134</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D56" s="4"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="2" t="s">
-        <x:v>135</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B57" s="3" t="s">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C57" s="4" t="s">
-        <x:v>137</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D57" s="4"/>
     </x:row>
     <x:row r="58" ht="28.5">
       <x:c r="A58" s="2" t="s">
-        <x:v>138</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B58" s="3" t="s">
-        <x:v>139</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C58" s="4" t="s">
-        <x:v>140</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D58" s="4"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="2" t="s">
-        <x:v>141</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B59" s="3" t="s">
-        <x:v>142</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C59" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D59" s="4"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="2" t="s">
-        <x:v>144</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B60" s="3" t="s">
-        <x:v>145</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C60" s="4" t="s">
-        <x:v>146</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D60" s="4"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="2" t="s">
-        <x:v>147</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B61" s="3" t="s">
-        <x:v>148</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C61" s="4" t="s">
-        <x:v>149</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D61" s="4"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2" t="s">
-        <x:v>150</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B62" s="3" t="s">
-        <x:v>151</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C62" s="4" t="s">
-        <x:v>152</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D62" s="4" t="s">
-        <x:v>153</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="s">
-        <x:v>154</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B63" s="6" t="s">
-        <x:v>155</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>156</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D63" s="7"/>
     </x:row>
@@ -3256,7 +3244,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20394abf4e74b18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd53a3a6df681450a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3271,56 +3259,56 @@
   <x:sheetData>
     <x:row r="1" ht="32.099998474121094" customHeight="1">
       <x:c r="A1" s="13" t="s">
-        <x:v>157</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B1" s="13"/>
     </x:row>
     <x:row r="3" ht="15">
       <x:c r="A3" s="8" t="s">
-        <x:v>158</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B3" s="9" t="s">
-        <x:v>159</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
       <x:c r="A4" s="8" t="s">
-        <x:v>160</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B4" s="9" t="s">
-        <x:v>161</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
       <x:c r="A5" s="8" t="s">
-        <x:v>162</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B5" s="9" t="s">
-        <x:v>163</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
       <x:c r="A6" s="8" t="s">
-        <x:v>164</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B6" s="9" t="s">
-        <x:v>165</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
       <x:c r="A7" s="8" t="s">
-        <x:v>166</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>167</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="10" t="s">
-        <x:v>168</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B9" s="10" t="s">
-        <x:v>169</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Remove persistent notification and update copy
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\Chat App - Local\outputs\app_strings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5342A9B4-A9EF-4419-B42B-58331CC47E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D421E606-F4A6-4F90-875D-C275F9A5E8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -467,9 +467,6 @@
     <t>notification_paused_body</t>
   </si>
   <si>
-    <t>File access is paused. Open the app to resume it.</t>
-  </si>
-  <si>
     <t>notification_pause_action</t>
   </si>
   <si>
@@ -1533,6 +1530,9 @@
   </si>
   <si>
     <t>Shown for a query without matches</t>
+  </si>
+  <si>
+    <t>Chat is paused. Open the app to resume it.</t>
   </si>
 </sst>
 </file>
@@ -2745,7 +2745,7 @@
         <v>147</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>148</v>
+        <v>503</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>142</v>
@@ -2754,232 +2754,232 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="C56" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>151</v>
       </c>
       <c r="D56" s="4"/>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="C57" s="4" t="s">
         <v>153</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>154</v>
       </c>
       <c r="D57" s="4"/>
     </row>
     <row r="58" spans="1:4" ht="28.5">
       <c r="A58" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="C58" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="D58" s="4"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="C59" s="4" t="s">
         <v>159</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>160</v>
       </c>
       <c r="D59" s="4"/>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="C60" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>163</v>
       </c>
       <c r="D60" s="4"/>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="C61" s="4" t="s">
         <v>165</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="D61" s="4"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B62" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="C62" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="D62" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="B63" s="6" t="s">
+      <c r="C63" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="C63" s="7" t="s">
-        <v>173</v>
       </c>
       <c r="D63" s="7"/>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B64" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="B64" s="13" t="s">
+      <c r="C64" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="C64" s="14" t="s">
-        <v>176</v>
       </c>
       <c r="D64" s="14"/>
     </row>
     <row r="65" spans="1:4" ht="28.5">
       <c r="A65" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="B65" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="C65" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C65" s="4" t="s">
-        <v>179</v>
-      </c>
       <c r="D65" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B66" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="B66" s="16" t="s">
+      <c r="C66" s="4" t="s">
         <v>181</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>182</v>
       </c>
       <c r="D66" s="4"/>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="B67" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="C67" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="D67" s="4"/>
     </row>
     <row r="68" spans="1:4" ht="28.5">
       <c r="A68" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B68" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="B68" s="16" t="s">
-        <v>187</v>
-      </c>
       <c r="C68" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D68" s="4"/>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B69" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="B69" s="16" t="s">
+      <c r="C69" s="4" t="s">
         <v>189</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>190</v>
       </c>
       <c r="D69" s="4"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B70" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="B70" s="16" t="s">
+      <c r="C70" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>193</v>
       </c>
       <c r="D70" s="4"/>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="B71" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="B71" s="16" t="s">
+      <c r="C71" s="4" t="s">
         <v>195</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>196</v>
       </c>
       <c r="D71" s="4"/>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B72" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="B72" s="16" t="s">
+      <c r="C72" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="D72" s="4" t="s">
         <v>199</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="B73" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="B73" s="16" t="s">
+      <c r="C73" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>203</v>
       </c>
       <c r="D73" s="4"/>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B74" s="16" t="s">
         <v>204</v>
-      </c>
-      <c r="B74" s="16" t="s">
-        <v>205</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>107</v>
@@ -2988,10 +2988,10 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B75" s="16" t="s">
         <v>206</v>
-      </c>
-      <c r="B75" s="16" t="s">
-        <v>207</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>107</v>
@@ -3000,1177 +3000,1177 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B76" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="B76" s="16" t="s">
+      <c r="C76" s="4" t="s">
         <v>209</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>210</v>
       </c>
       <c r="D76" s="4"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="B77" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="B77" s="16" t="s">
+      <c r="C77" s="4" t="s">
         <v>212</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>213</v>
       </c>
       <c r="D77" s="4"/>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="B78" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="B78" s="16" t="s">
+      <c r="C78" s="4" t="s">
         <v>215</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>216</v>
       </c>
       <c r="D78" s="4"/>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="B79" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="B79" s="16" t="s">
+      <c r="C79" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="D79" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B80" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="B80" s="18" t="s">
-        <v>222</v>
-      </c>
       <c r="C80" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D80" s="7"/>
     </row>
     <row r="81" spans="1:4" ht="14.25" customHeight="1">
       <c r="A81" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="B81" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="B81" s="21" t="s">
+      <c r="C81" s="23" t="s">
         <v>224</v>
       </c>
-      <c r="C81" s="23" t="s">
+      <c r="D81" s="23" t="s">
         <v>225</v>
-      </c>
-      <c r="D81" s="23" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="14.25" customHeight="1">
       <c r="A82" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="B82" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="B82" s="21" t="s">
+      <c r="C82" s="23" t="s">
         <v>228</v>
       </c>
-      <c r="C82" s="23" t="s">
-        <v>229</v>
-      </c>
       <c r="D82" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="14.25" customHeight="1">
       <c r="A83" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="B83" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="B83" s="21" t="s">
+      <c r="C83" s="23" t="s">
         <v>231</v>
       </c>
-      <c r="C83" s="23" t="s">
-        <v>232</v>
-      </c>
       <c r="D83" s="23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="14.25" customHeight="1">
       <c r="A84" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="B84" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="B84" s="21" t="s">
+      <c r="C84" s="23" t="s">
         <v>234</v>
-      </c>
-      <c r="C84" s="23" t="s">
-        <v>235</v>
       </c>
       <c r="D84" s="23"/>
     </row>
     <row r="85" spans="1:4" ht="14.25" customHeight="1">
       <c r="A85" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="B85" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="B85" s="21" t="s">
+      <c r="C85" s="23" t="s">
         <v>237</v>
-      </c>
-      <c r="C85" s="23" t="s">
-        <v>238</v>
       </c>
       <c r="D85" s="23"/>
     </row>
     <row r="86" spans="1:4" ht="14.25" customHeight="1">
       <c r="A86" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="B86" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="B86" s="21" t="s">
+      <c r="C86" s="23" t="s">
         <v>240</v>
-      </c>
-      <c r="C86" s="23" t="s">
-        <v>241</v>
       </c>
       <c r="D86" s="23"/>
     </row>
     <row r="87" spans="1:4" ht="14.25" customHeight="1">
       <c r="A87" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B87" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="B87" s="21" t="s">
-        <v>243</v>
-      </c>
       <c r="C87" s="23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D87" s="23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="26.45" customHeight="1">
       <c r="A88" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B88" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="B88" s="21" t="s">
+      <c r="C88" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="C88" s="23" t="s">
+      <c r="D88" s="23" t="s">
         <v>246</v>
-      </c>
-      <c r="D88" s="23" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="14.25" customHeight="1">
       <c r="A89" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B89" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="B89" s="21" t="s">
+      <c r="C89" s="23" t="s">
         <v>249</v>
-      </c>
-      <c r="C89" s="23" t="s">
-        <v>250</v>
       </c>
       <c r="D89" s="23"/>
     </row>
     <row r="90" spans="1:4" ht="14.25" customHeight="1">
       <c r="A90" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="B90" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="B90" s="21" t="s">
-        <v>252</v>
-      </c>
       <c r="C90" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D90" s="23"/>
     </row>
     <row r="91" spans="1:4" ht="14.25" customHeight="1">
       <c r="A91" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B91" s="21" t="s">
         <v>253</v>
       </c>
-      <c r="B91" s="21" t="s">
-        <v>254</v>
-      </c>
       <c r="C91" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D91" s="23"/>
     </row>
     <row r="92" spans="1:4" ht="14.25" customHeight="1">
       <c r="A92" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="B92" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="B92" s="21" t="s">
-        <v>256</v>
-      </c>
       <c r="C92" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D92" s="23"/>
     </row>
     <row r="93" spans="1:4" ht="14.25" customHeight="1">
       <c r="A93" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="B93" s="22" t="s">
         <v>257</v>
       </c>
-      <c r="B93" s="22" t="s">
+      <c r="C93" s="24" t="s">
         <v>258</v>
-      </c>
-      <c r="C93" s="24" t="s">
-        <v>259</v>
       </c>
       <c r="D93" s="24"/>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="26" t="s">
+        <v>259</v>
+      </c>
+      <c r="B94" s="29" t="s">
         <v>260</v>
       </c>
-      <c r="B94" s="29" t="s">
+      <c r="C94" s="32" t="s">
         <v>261</v>
-      </c>
-      <c r="C94" s="32" t="s">
-        <v>262</v>
       </c>
       <c r="D94" s="32"/>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="B95" s="30" t="s">
         <v>263</v>
       </c>
-      <c r="B95" s="30" t="s">
+      <c r="C95" s="33" t="s">
         <v>264</v>
       </c>
-      <c r="C95" s="33" t="s">
+      <c r="D95" s="33" t="s">
         <v>265</v>
-      </c>
-      <c r="D95" s="33" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="27" t="s">
+        <v>266</v>
+      </c>
+      <c r="B96" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="B96" s="30" t="s">
+      <c r="C96" s="34" t="s">
         <v>268</v>
-      </c>
-      <c r="C96" s="34" t="s">
-        <v>269</v>
       </c>
       <c r="D96" s="34"/>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="B97" s="30" t="s">
         <v>270</v>
       </c>
-      <c r="B97" s="30" t="s">
+      <c r="C97" s="33" t="s">
         <v>271</v>
-      </c>
-      <c r="C97" s="33" t="s">
-        <v>272</v>
       </c>
       <c r="D97" s="33"/>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="B98" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="B98" s="30" t="s">
+      <c r="C98" s="34" t="s">
         <v>274</v>
-      </c>
-      <c r="C98" s="34" t="s">
-        <v>275</v>
       </c>
       <c r="D98" s="34"/>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="27" t="s">
+        <v>275</v>
+      </c>
+      <c r="B99" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="B99" s="30" t="s">
+      <c r="C99" s="33" t="s">
         <v>277</v>
-      </c>
-      <c r="C99" s="33" t="s">
-        <v>278</v>
       </c>
       <c r="D99" s="33"/>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="B100" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="B100" s="30" t="s">
+      <c r="C100" s="34" t="s">
         <v>280</v>
-      </c>
-      <c r="C100" s="34" t="s">
-        <v>281</v>
       </c>
       <c r="D100" s="34"/>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="B101" s="30" t="s">
         <v>282</v>
       </c>
-      <c r="B101" s="30" t="s">
+      <c r="C101" s="33" t="s">
         <v>283</v>
-      </c>
-      <c r="C101" s="33" t="s">
-        <v>284</v>
       </c>
       <c r="D101" s="33"/>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="B102" s="30" t="s">
         <v>285</v>
       </c>
-      <c r="B102" s="30" t="s">
+      <c r="C102" s="34" t="s">
         <v>286</v>
-      </c>
-      <c r="C102" s="34" t="s">
-        <v>287</v>
       </c>
       <c r="D102" s="34"/>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="27" t="s">
+        <v>287</v>
+      </c>
+      <c r="B103" s="30" t="s">
         <v>288</v>
       </c>
-      <c r="B103" s="30" t="s">
+      <c r="C103" s="33" t="s">
         <v>289</v>
-      </c>
-      <c r="C103" s="33" t="s">
-        <v>290</v>
       </c>
       <c r="D103" s="33"/>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="27" t="s">
+        <v>290</v>
+      </c>
+      <c r="B104" s="30" t="s">
         <v>291</v>
       </c>
-      <c r="B104" s="30" t="s">
+      <c r="C104" s="34" t="s">
         <v>292</v>
-      </c>
-      <c r="C104" s="34" t="s">
-        <v>293</v>
       </c>
       <c r="D104" s="34"/>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="27" t="s">
+        <v>293</v>
+      </c>
+      <c r="B105" s="30" t="s">
         <v>294</v>
       </c>
-      <c r="B105" s="30" t="s">
+      <c r="C105" s="33" t="s">
         <v>295</v>
-      </c>
-      <c r="C105" s="33" t="s">
-        <v>296</v>
       </c>
       <c r="D105" s="33"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="B106" s="30" t="s">
         <v>297</v>
       </c>
-      <c r="B106" s="30" t="s">
-        <v>298</v>
-      </c>
       <c r="C106" s="34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D106" s="34"/>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="27" t="s">
+        <v>298</v>
+      </c>
+      <c r="B107" s="30" t="s">
         <v>299</v>
       </c>
-      <c r="B107" s="30" t="s">
+      <c r="C107" s="33" t="s">
         <v>300</v>
-      </c>
-      <c r="C107" s="33" t="s">
-        <v>301</v>
       </c>
       <c r="D107" s="33"/>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="B108" s="30" t="s">
         <v>302</v>
       </c>
-      <c r="B108" s="30" t="s">
+      <c r="C108" s="34" t="s">
         <v>303</v>
-      </c>
-      <c r="C108" s="34" t="s">
-        <v>304</v>
       </c>
       <c r="D108" s="34"/>
     </row>
     <row r="109" spans="1:4" ht="28.5">
       <c r="A109" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="B109" s="30" t="s">
         <v>305</v>
       </c>
-      <c r="B109" s="30" t="s">
+      <c r="C109" s="33" t="s">
         <v>306</v>
-      </c>
-      <c r="C109" s="33" t="s">
-        <v>307</v>
       </c>
       <c r="D109" s="33"/>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="B110" s="30" t="s">
         <v>308</v>
       </c>
-      <c r="B110" s="30" t="s">
+      <c r="C110" s="34" t="s">
         <v>309</v>
-      </c>
-      <c r="C110" s="34" t="s">
-        <v>310</v>
       </c>
       <c r="D110" s="34"/>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="B111" s="30" t="s">
         <v>311</v>
       </c>
-      <c r="B111" s="30" t="s">
+      <c r="C111" s="33" t="s">
         <v>312</v>
-      </c>
-      <c r="C111" s="33" t="s">
-        <v>313</v>
       </c>
       <c r="D111" s="33"/>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="B112" s="31" t="s">
         <v>314</v>
       </c>
-      <c r="B112" s="31" t="s">
+      <c r="C112" s="35" t="s">
         <v>315</v>
-      </c>
-      <c r="C112" s="35" t="s">
-        <v>316</v>
       </c>
       <c r="D112" s="35"/>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" t="s">
+        <v>316</v>
+      </c>
+      <c r="B113" t="s">
         <v>317</v>
       </c>
-      <c r="B113" t="s">
+      <c r="C113" t="s">
         <v>318</v>
-      </c>
-      <c r="C113" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" t="s">
+        <v>319</v>
+      </c>
+      <c r="B114" t="s">
         <v>320</v>
       </c>
-      <c r="B114" t="s">
-        <v>321</v>
-      </c>
       <c r="C114" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" t="s">
+        <v>321</v>
+      </c>
+      <c r="B115" t="s">
         <v>322</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C115" t="s">
         <v>323</v>
       </c>
-      <c r="C115" t="s">
+      <c r="D115" t="s">
         <v>324</v>
-      </c>
-      <c r="D115" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" t="s">
+        <v>325</v>
+      </c>
+      <c r="B116" t="s">
         <v>326</v>
       </c>
-      <c r="B116" t="s">
+      <c r="C116" t="s">
         <v>327</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
         <v>328</v>
-      </c>
-      <c r="D116" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" t="s">
+        <v>329</v>
+      </c>
+      <c r="B117" t="s">
         <v>330</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C117" t="s">
         <v>331</v>
-      </c>
-      <c r="C117" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="36" t="s">
+        <v>332</v>
+      </c>
+      <c r="B118" s="39" t="s">
         <v>333</v>
       </c>
-      <c r="B118" s="39" t="s">
+      <c r="C118" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="C118" s="25" t="s">
+      <c r="D118" s="25" t="s">
         <v>335</v>
-      </c>
-      <c r="D118" s="25" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="37" t="s">
+        <v>336</v>
+      </c>
+      <c r="B119" s="40" t="s">
         <v>337</v>
       </c>
-      <c r="B119" s="40" t="s">
+      <c r="C119" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="D119" s="11" t="s">
         <v>338</v>
-      </c>
-      <c r="C119" s="11" t="s">
-        <v>335</v>
-      </c>
-      <c r="D119" s="11" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="37" t="s">
+        <v>339</v>
+      </c>
+      <c r="B120" s="40" t="s">
         <v>340</v>
       </c>
-      <c r="B120" s="40" t="s">
+      <c r="C120" s="11" t="s">
         <v>341</v>
       </c>
-      <c r="C120" s="11" t="s">
+      <c r="D120" s="11" t="s">
         <v>342</v>
-      </c>
-      <c r="D120" s="11" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="28.5">
       <c r="A121" s="37" t="s">
+        <v>343</v>
+      </c>
+      <c r="B121" s="40" t="s">
         <v>344</v>
       </c>
-      <c r="B121" s="40" t="s">
+      <c r="C121" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="C121" s="11" t="s">
+      <c r="D121" s="11" t="s">
         <v>346</v>
-      </c>
-      <c r="D121" s="11" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="28.5">
       <c r="A122" s="37" t="s">
+        <v>347</v>
+      </c>
+      <c r="B122" s="40" t="s">
         <v>348</v>
       </c>
-      <c r="B122" s="40" t="s">
+      <c r="C122" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="C122" s="11" t="s">
+      <c r="D122" s="11" t="s">
         <v>350</v>
-      </c>
-      <c r="D122" s="11" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="37" t="s">
+        <v>351</v>
+      </c>
+      <c r="B123" s="40" t="s">
         <v>352</v>
       </c>
-      <c r="B123" s="40" t="s">
+      <c r="C123" s="11" t="s">
         <v>353</v>
-      </c>
-      <c r="C123" s="11" t="s">
-        <v>354</v>
       </c>
       <c r="D123" s="11"/>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="37" t="s">
+        <v>354</v>
+      </c>
+      <c r="B124" s="40" t="s">
         <v>355</v>
       </c>
-      <c r="B124" s="40" t="s">
+      <c r="C124" s="11" t="s">
         <v>356</v>
-      </c>
-      <c r="C124" s="11" t="s">
-        <v>357</v>
       </c>
       <c r="D124" s="11"/>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="37" t="s">
+        <v>357</v>
+      </c>
+      <c r="B125" s="40" t="s">
         <v>358</v>
       </c>
-      <c r="B125" s="40" t="s">
+      <c r="C125" s="11" t="s">
         <v>359</v>
-      </c>
-      <c r="C125" s="11" t="s">
-        <v>360</v>
       </c>
       <c r="D125" s="11"/>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="37" t="s">
+        <v>360</v>
+      </c>
+      <c r="B126" s="40" t="s">
         <v>361</v>
       </c>
-      <c r="B126" s="40" t="s">
+      <c r="C126" s="11" t="s">
         <v>362</v>
-      </c>
-      <c r="C126" s="11" t="s">
-        <v>363</v>
       </c>
       <c r="D126" s="11"/>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="37" t="s">
+        <v>363</v>
+      </c>
+      <c r="B127" s="40" t="s">
         <v>364</v>
       </c>
-      <c r="B127" s="40" t="s">
-        <v>365</v>
-      </c>
       <c r="C127" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D127" s="11"/>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="37" t="s">
+        <v>365</v>
+      </c>
+      <c r="B128" s="40" t="s">
         <v>366</v>
       </c>
-      <c r="B128" s="40" t="s">
-        <v>367</v>
-      </c>
       <c r="C128" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D128" s="11"/>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="37" t="s">
+        <v>367</v>
+      </c>
+      <c r="B129" s="40" t="s">
         <v>368</v>
       </c>
-      <c r="B129" s="40" t="s">
-        <v>369</v>
-      </c>
       <c r="C129" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D129" s="11"/>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="37" t="s">
+        <v>369</v>
+      </c>
+      <c r="B130" s="40" t="s">
         <v>370</v>
       </c>
-      <c r="B130" s="40" t="s">
-        <v>371</v>
-      </c>
       <c r="C130" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D130" s="11"/>
     </row>
     <row r="131" spans="1:4" ht="28.5">
       <c r="A131" s="37" t="s">
+        <v>371</v>
+      </c>
+      <c r="B131" s="40" t="s">
         <v>372</v>
       </c>
-      <c r="B131" s="40" t="s">
+      <c r="C131" s="11" t="s">
         <v>373</v>
-      </c>
-      <c r="C131" s="11" t="s">
-        <v>374</v>
       </c>
       <c r="D131" s="11"/>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="37" t="s">
+        <v>374</v>
+      </c>
+      <c r="B132" s="40" t="s">
         <v>375</v>
       </c>
-      <c r="B132" s="40" t="s">
+      <c r="C132" s="11" t="s">
         <v>376</v>
-      </c>
-      <c r="C132" s="11" t="s">
-        <v>377</v>
       </c>
       <c r="D132" s="11"/>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="37" t="s">
+        <v>377</v>
+      </c>
+      <c r="B133" s="40" t="s">
         <v>378</v>
       </c>
-      <c r="B133" s="40" t="s">
+      <c r="C133" s="11" t="s">
         <v>379</v>
-      </c>
-      <c r="C133" s="11" t="s">
-        <v>380</v>
       </c>
       <c r="D133" s="11"/>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="37" t="s">
+        <v>380</v>
+      </c>
+      <c r="B134" s="40" t="s">
         <v>381</v>
       </c>
-      <c r="B134" s="40" t="s">
+      <c r="C134" s="11" t="s">
         <v>382</v>
-      </c>
-      <c r="C134" s="11" t="s">
-        <v>383</v>
       </c>
       <c r="D134" s="11"/>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="38" t="s">
+        <v>383</v>
+      </c>
+      <c r="B135" s="41" t="s">
         <v>384</v>
       </c>
-      <c r="B135" s="41" t="s">
-        <v>385</v>
-      </c>
       <c r="C135" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D135" s="14"/>
     </row>
     <row r="136" spans="1:4" ht="28.5">
       <c r="A136" s="42" t="s">
+        <v>385</v>
+      </c>
+      <c r="B136" s="44" t="s">
         <v>386</v>
       </c>
-      <c r="B136" s="44" t="s">
+      <c r="C136" s="14" t="s">
         <v>387</v>
       </c>
-      <c r="C136" s="14" t="s">
+      <c r="D136" s="14" t="s">
         <v>388</v>
-      </c>
-      <c r="D136" s="14" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="43" t="s">
+        <v>389</v>
+      </c>
+      <c r="B137" s="45" t="s">
         <v>390</v>
       </c>
-      <c r="B137" s="45" t="s">
+      <c r="C137" s="4" t="s">
         <v>391</v>
-      </c>
-      <c r="C137" s="4" t="s">
-        <v>392</v>
       </c>
       <c r="D137" s="4"/>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="43" t="s">
+        <v>392</v>
+      </c>
+      <c r="B138" s="45" t="s">
         <v>393</v>
       </c>
-      <c r="B138" s="45" t="s">
+      <c r="C138" s="4" t="s">
         <v>394</v>
-      </c>
-      <c r="C138" s="4" t="s">
-        <v>395</v>
       </c>
       <c r="D138" s="4"/>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="43" t="s">
+        <v>395</v>
+      </c>
+      <c r="B139" s="45" t="s">
         <v>396</v>
       </c>
-      <c r="B139" s="45" t="s">
-        <v>397</v>
-      </c>
       <c r="C139" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D139" s="4"/>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="43" t="s">
+        <v>397</v>
+      </c>
+      <c r="B140" s="45" t="s">
         <v>398</v>
       </c>
-      <c r="B140" s="45" t="s">
-        <v>399</v>
-      </c>
       <c r="C140" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D140" s="4"/>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="43" t="s">
+        <v>399</v>
+      </c>
+      <c r="B141" s="45" t="s">
         <v>400</v>
       </c>
-      <c r="B141" s="45" t="s">
+      <c r="C141" s="4" t="s">
         <v>401</v>
-      </c>
-      <c r="C141" s="4" t="s">
-        <v>402</v>
       </c>
       <c r="D141" s="4"/>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="43" t="s">
+        <v>402</v>
+      </c>
+      <c r="B142" s="45" t="s">
         <v>403</v>
       </c>
-      <c r="B142" s="45" t="s">
+      <c r="C142" s="4" t="s">
         <v>404</v>
-      </c>
-      <c r="C142" s="4" t="s">
-        <v>405</v>
       </c>
       <c r="D142" s="4"/>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="43" t="s">
+        <v>405</v>
+      </c>
+      <c r="B143" s="45" t="s">
         <v>406</v>
       </c>
-      <c r="B143" s="45" t="s">
-        <v>407</v>
-      </c>
       <c r="C143" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D143" s="4"/>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="43" t="s">
+        <v>407</v>
+      </c>
+      <c r="B144" s="45" t="s">
         <v>408</v>
       </c>
-      <c r="B144" s="45" t="s">
+      <c r="C144" s="4" t="s">
         <v>409</v>
-      </c>
-      <c r="C144" s="4" t="s">
-        <v>410</v>
       </c>
       <c r="D144" s="4"/>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="43" t="s">
+        <v>410</v>
+      </c>
+      <c r="B145" s="45" t="s">
         <v>411</v>
       </c>
-      <c r="B145" s="45" t="s">
+      <c r="C145" s="4" t="s">
         <v>412</v>
-      </c>
-      <c r="C145" s="4" t="s">
-        <v>413</v>
       </c>
       <c r="D145" s="4"/>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="43" t="s">
+        <v>413</v>
+      </c>
+      <c r="B146" s="45" t="s">
         <v>414</v>
       </c>
-      <c r="B146" s="45" t="s">
+      <c r="C146" s="4" t="s">
         <v>415</v>
-      </c>
-      <c r="C146" s="4" t="s">
-        <v>416</v>
       </c>
       <c r="D146" s="4"/>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="43" t="s">
+        <v>416</v>
+      </c>
+      <c r="B147" s="45" t="s">
         <v>417</v>
       </c>
-      <c r="B147" s="45" t="s">
+      <c r="C147" s="4" t="s">
         <v>418</v>
-      </c>
-      <c r="C147" s="4" t="s">
-        <v>419</v>
       </c>
       <c r="D147" s="4"/>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="43" t="s">
+        <v>419</v>
+      </c>
+      <c r="B148" s="45" t="s">
         <v>420</v>
       </c>
-      <c r="B148" s="45" t="s">
+      <c r="C148" s="4" t="s">
         <v>421</v>
-      </c>
-      <c r="C148" s="4" t="s">
-        <v>422</v>
       </c>
       <c r="D148" s="4"/>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="43" t="s">
+        <v>422</v>
+      </c>
+      <c r="B149" s="45" t="s">
         <v>423</v>
       </c>
-      <c r="B149" s="45" t="s">
+      <c r="C149" s="4" t="s">
         <v>424</v>
-      </c>
-      <c r="C149" s="4" t="s">
-        <v>425</v>
       </c>
       <c r="D149" s="4"/>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="43" t="s">
+        <v>425</v>
+      </c>
+      <c r="B150" s="45" t="s">
         <v>426</v>
       </c>
-      <c r="B150" s="45" t="s">
+      <c r="C150" s="4" t="s">
         <v>427</v>
-      </c>
-      <c r="C150" s="4" t="s">
-        <v>428</v>
       </c>
       <c r="D150" s="4"/>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="43" t="s">
+        <v>428</v>
+      </c>
+      <c r="B151" s="45" t="s">
+        <v>428</v>
+      </c>
+      <c r="C151" s="4" t="s">
         <v>429</v>
-      </c>
-      <c r="B151" s="45" t="s">
-        <v>429</v>
-      </c>
-      <c r="C151" s="4" t="s">
-        <v>430</v>
       </c>
       <c r="D151" s="4"/>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="43" t="s">
+        <v>430</v>
+      </c>
+      <c r="B152" s="45" t="s">
         <v>431</v>
       </c>
-      <c r="B152" s="45" t="s">
+      <c r="C152" s="4" t="s">
         <v>432</v>
-      </c>
-      <c r="C152" s="4" t="s">
-        <v>433</v>
       </c>
       <c r="D152" s="4"/>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" t="s">
+        <v>433</v>
+      </c>
+      <c r="B153" t="s">
         <v>434</v>
       </c>
-      <c r="B153" t="s">
+      <c r="C153" t="s">
         <v>435</v>
-      </c>
-      <c r="C153" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" t="s">
+        <v>436</v>
+      </c>
+      <c r="B154" t="s">
         <v>437</v>
       </c>
-      <c r="B154" t="s">
-        <v>438</v>
-      </c>
       <c r="C154" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" t="s">
+        <v>438</v>
+      </c>
+      <c r="B155" t="s">
         <v>439</v>
       </c>
-      <c r="B155" t="s">
-        <v>440</v>
-      </c>
       <c r="C155" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" t="s">
+        <v>440</v>
+      </c>
+      <c r="B156" t="s">
         <v>441</v>
       </c>
-      <c r="B156" t="s">
-        <v>442</v>
-      </c>
       <c r="C156" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" t="s">
+        <v>442</v>
+      </c>
+      <c r="B157" t="s">
         <v>443</v>
       </c>
-      <c r="B157" t="s">
-        <v>444</v>
-      </c>
       <c r="C157" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" t="s">
+        <v>444</v>
+      </c>
+      <c r="B158" t="s">
         <v>445</v>
       </c>
-      <c r="B158" t="s">
+      <c r="C158" t="s">
         <v>446</v>
-      </c>
-      <c r="C158" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="159" spans="1:4" ht="20.100000000000001" customHeight="1">
       <c r="A159" s="46" t="s">
+        <v>447</v>
+      </c>
+      <c r="B159" s="47" t="s">
         <v>448</v>
       </c>
-      <c r="B159" s="47" t="s">
+      <c r="C159" s="48" t="s">
         <v>449</v>
-      </c>
-      <c r="C159" s="48" t="s">
-        <v>450</v>
       </c>
       <c r="D159" s="4"/>
     </row>
     <row r="160" spans="1:4" ht="20.100000000000001" customHeight="1">
       <c r="A160" s="46" t="s">
+        <v>450</v>
+      </c>
+      <c r="B160" s="47" t="s">
         <v>451</v>
       </c>
-      <c r="B160" s="47" t="s">
+      <c r="C160" s="48" t="s">
         <v>452</v>
       </c>
-      <c r="C160" s="48" t="s">
+      <c r="D160" s="4" t="s">
         <v>453</v>
-      </c>
-      <c r="D160" s="4" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" t="s">
+        <v>454</v>
+      </c>
+      <c r="B161" t="s">
         <v>455</v>
       </c>
-      <c r="B161" t="s">
-        <v>456</v>
-      </c>
       <c r="C161" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" t="s">
+        <v>456</v>
+      </c>
+      <c r="B162" t="s">
         <v>457</v>
       </c>
-      <c r="B162" t="s">
-        <v>458</v>
-      </c>
       <c r="C162" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" t="s">
+        <v>458</v>
+      </c>
+      <c r="B163" t="s">
         <v>459</v>
       </c>
-      <c r="B163" t="s">
+      <c r="C163" t="s">
         <v>460</v>
-      </c>
-      <c r="C163" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" t="s">
+        <v>461</v>
+      </c>
+      <c r="B164" t="s">
         <v>462</v>
       </c>
-      <c r="B164" t="s">
-        <v>463</v>
-      </c>
       <c r="C164" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" t="s">
+        <v>463</v>
+      </c>
+      <c r="B165" t="s">
         <v>464</v>
       </c>
-      <c r="B165" t="s">
-        <v>465</v>
-      </c>
       <c r="C165" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" t="s">
+        <v>465</v>
+      </c>
+      <c r="B166" t="s">
         <v>466</v>
       </c>
-      <c r="B166" t="s">
-        <v>467</v>
-      </c>
       <c r="C166" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" t="s">
+        <v>467</v>
+      </c>
+      <c r="B167" t="s">
         <v>468</v>
       </c>
-      <c r="B167" t="s">
-        <v>469</v>
-      </c>
       <c r="C167" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" t="s">
+        <v>469</v>
+      </c>
+      <c r="B168" t="s">
         <v>470</v>
       </c>
-      <c r="B168" t="s">
-        <v>471</v>
-      </c>
       <c r="C168" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" t="s">
+        <v>471</v>
+      </c>
+      <c r="B169" t="s">
         <v>472</v>
       </c>
-      <c r="B169" t="s">
+      <c r="C169" t="s">
         <v>473</v>
-      </c>
-      <c r="C169" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" t="s">
+        <v>474</v>
+      </c>
+      <c r="B170" t="s">
         <v>475</v>
-      </c>
-      <c r="B170" t="s">
-        <v>476</v>
       </c>
       <c r="C170" t="s">
         <v>30</v>
       </c>
       <c r="D170" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" t="s">
+        <v>477</v>
+      </c>
+      <c r="B171" t="s">
         <v>478</v>
-      </c>
-      <c r="B171" t="s">
-        <v>479</v>
       </c>
       <c r="C171" t="s">
         <v>30</v>
       </c>
       <c r="D171" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B172" t="s">
         <v>34</v>
@@ -4179,119 +4179,119 @@
         <v>30</v>
       </c>
       <c r="D172" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" t="s">
+        <v>481</v>
+      </c>
+      <c r="B173" t="s">
         <v>482</v>
-      </c>
-      <c r="B173" t="s">
-        <v>483</v>
       </c>
       <c r="C173" t="s">
         <v>30</v>
       </c>
       <c r="D173" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" t="s">
+        <v>484</v>
+      </c>
+      <c r="B174" t="s">
         <v>485</v>
-      </c>
-      <c r="B174" t="s">
-        <v>486</v>
       </c>
       <c r="C174" t="s">
         <v>30</v>
       </c>
       <c r="D174" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" t="s">
+        <v>486</v>
+      </c>
+      <c r="B175" t="s">
         <v>487</v>
       </c>
-      <c r="B175" t="s">
+      <c r="C175" t="s">
         <v>488</v>
       </c>
-      <c r="C175" t="s">
+      <c r="D175" t="s">
         <v>489</v>
-      </c>
-      <c r="D175" t="s">
-        <v>490</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" t="s">
+        <v>490</v>
+      </c>
+      <c r="B176" t="s">
         <v>491</v>
       </c>
-      <c r="B176" t="s">
+      <c r="C176" t="s">
+        <v>488</v>
+      </c>
+      <c r="D176" t="s">
         <v>492</v>
-      </c>
-      <c r="C176" t="s">
-        <v>489</v>
-      </c>
-      <c r="D176" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" t="s">
+        <v>493</v>
+      </c>
+      <c r="B177" t="s">
         <v>494</v>
       </c>
-      <c r="B177" t="s">
-        <v>495</v>
-      </c>
       <c r="C177" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D177" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" t="s">
+        <v>495</v>
+      </c>
+      <c r="B178" t="s">
         <v>496</v>
       </c>
-      <c r="B178" t="s">
-        <v>497</v>
-      </c>
       <c r="C178" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D178" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" t="s">
+        <v>497</v>
+      </c>
+      <c r="B179" t="s">
         <v>498</v>
       </c>
-      <c r="B179" t="s">
+      <c r="C179" t="s">
+        <v>488</v>
+      </c>
+      <c r="D179" t="s">
         <v>499</v>
-      </c>
-      <c r="C179" t="s">
-        <v>489</v>
-      </c>
-      <c r="D179" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="180" spans="1:4">
       <c r="A180" t="s">
+        <v>500</v>
+      </c>
+      <c r="B180" t="s">
         <v>501</v>
       </c>
-      <c r="B180" t="s">
+      <c r="C180" t="s">
+        <v>488</v>
+      </c>
+      <c r="D180" t="s">
         <v>502</v>
-      </c>
-      <c r="C180" t="s">
-        <v>489</v>
-      </c>
-      <c r="D180" t="s">
-        <v>503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep Test App release naming
</commit_message>
<xml_diff>
--- a/outputs/app_strings/app_strings.xlsx
+++ b/outputs/app_strings/app_strings.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="R76ef54ec72ac4f27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="Rf44f7e5b2f4c42d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android Strings" sheetId="1" r:id="R2d81344bf1624be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" r:id="R956649b817f14457"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -237,9 +237,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">update_ready_body</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Between %1$s is ready. Download the APK from GitHub and install it over this app. Your local messages will stay on this phone.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Update dialog body</x:t>
@@ -2421,1711 +2418,1711 @@
       <x:c r="A32" s="2" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B32" s="3" t="s">
+      <x:c r="B32" s="3" t="str">
+        <x:v>Test App %1$s is ready. Download the APK from GitHub and install it over this app. Your local messages will stay on this phone.</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="C32" s="4" t="s">
+      <x:c r="D32" s="4" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="D32" s="4" t="s">
-        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="2" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B33" s="3" t="s">
+      <x:c r="C33" s="4" t="s">
         <x:v>80</x:v>
-      </x:c>
-      <x:c r="C33" s="4" t="s">
-        <x:v>81</x:v>
       </x:c>
       <x:c r="D33" s="4"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="2" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B34" s="3" t="s">
-        <x:v>83</x:v>
-      </x:c>
       <x:c r="C34" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D34" s="4"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="2" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B35" s="3" t="s">
+      <x:c r="C35" s="4" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="C35" s="4" t="s">
-        <x:v>86</x:v>
       </x:c>
       <x:c r="D35" s="4"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="2" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B36" s="3" t="s">
+      <x:c r="C36" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="C36" s="4" t="s">
-        <x:v>89</x:v>
       </x:c>
       <x:c r="D36" s="4"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="2" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B37" s="3" t="s">
+      <x:c r="C37" s="4" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="C37" s="4" t="s">
-        <x:v>92</x:v>
       </x:c>
       <x:c r="D37" s="4"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C38" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D38" s="4"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="2" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="B39" s="3" t="s">
-        <x:v>96</x:v>
-      </x:c>
       <x:c r="C39" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D39" s="4"/>
     </x:row>
     <x:row r="40" ht="28.5">
       <x:c r="A40" s="2" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="B40" s="3" t="s">
+      <x:c r="C40" s="4" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="C40" s="4" t="s">
-        <x:v>99</x:v>
       </x:c>
       <x:c r="D40" s="4"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B41" s="3" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="B41" s="3" t="s">
+      <x:c r="C41" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="C41" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
       <x:c r="D41" s="4"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B42" s="3" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="B42" s="3" t="s">
+      <x:c r="C42" s="4" t="s">
         <x:v>104</x:v>
-      </x:c>
-      <x:c r="C42" s="4" t="s">
-        <x:v>105</x:v>
       </x:c>
       <x:c r="D42" s="4"/>
     </x:row>
     <x:row r="43" ht="28.5">
       <x:c r="A43" s="2" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B43" s="3" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="B43" s="3" t="s">
-        <x:v>107</x:v>
-      </x:c>
       <x:c r="C43" s="4" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D43" s="4"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B44" s="3" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="B44" s="3" t="s">
+      <x:c r="C44" s="4" t="s">
         <x:v>109</x:v>
-      </x:c>
-      <x:c r="C44" s="4" t="s">
-        <x:v>110</x:v>
       </x:c>
       <x:c r="D44" s="4"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="2" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B45" s="3" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="B45" s="3" t="s">
+      <x:c r="C45" s="4" t="s">
         <x:v>112</x:v>
-      </x:c>
-      <x:c r="C45" s="4" t="s">
-        <x:v>113</x:v>
       </x:c>
       <x:c r="D45" s="4"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="2" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="B46" s="3" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="B46" s="3" t="s">
-        <x:v>115</x:v>
-      </x:c>
       <x:c r="C46" s="4" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D46" s="4"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="B47" s="3" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="B47" s="3" t="s">
-        <x:v>117</x:v>
-      </x:c>
       <x:c r="C47" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D47" s="4"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B48" s="3" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="B48" s="3" t="s">
-        <x:v>119</x:v>
-      </x:c>
       <x:c r="C48" s="4" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D48" s="4"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="B49" s="3" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="B49" s="3" t="s">
-        <x:v>121</x:v>
-      </x:c>
       <x:c r="C49" s="4" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D49" s="4"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="2" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B50" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="B50" s="3" t="s">
+      <x:c r="C50" s="4" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="C50" s="4" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="D50" s="4"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="B51" s="3" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="B51" s="3" t="s">
-        <x:v>126</x:v>
-      </x:c>
       <x:c r="C51" s="4" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D51" s="4"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="2" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="B52" s="3" t="s">
+      <x:c r="C52" s="4" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="C52" s="4" t="s">
-        <x:v>129</x:v>
       </x:c>
       <x:c r="D52" s="4"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="B53" s="3" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="B53" s="3" t="s">
-        <x:v>131</x:v>
-      </x:c>
       <x:c r="C53" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D53" s="4"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B54" s="3" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="B54" s="3" t="s">
-        <x:v>133</x:v>
-      </x:c>
       <x:c r="C54" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D54" s="4"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="2" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="B55" s="3" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="B55" s="3" t="s">
-        <x:v>135</x:v>
-      </x:c>
       <x:c r="C55" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D55" s="4"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="2" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="B56" s="3" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="B56" s="3" t="s">
+      <x:c r="C56" s="4" t="s">
         <x:v>137</x:v>
-      </x:c>
-      <x:c r="C56" s="4" t="s">
-        <x:v>138</x:v>
       </x:c>
       <x:c r="D56" s="4"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="2" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="B57" s="3" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="B57" s="3" t="s">
+      <x:c r="C57" s="4" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="C57" s="4" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="D57" s="4"/>
     </x:row>
     <x:row r="58" ht="28.5">
       <x:c r="A58" s="2" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B58" s="3" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="B58" s="3" t="s">
+      <x:c r="C58" s="4" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="C58" s="4" t="s">
-        <x:v>144</x:v>
       </x:c>
       <x:c r="D58" s="4"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="2" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="B59" s="3" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="B59" s="3" t="s">
+      <x:c r="C59" s="4" t="s">
         <x:v>146</x:v>
-      </x:c>
-      <x:c r="C59" s="4" t="s">
-        <x:v>147</x:v>
       </x:c>
       <x:c r="D59" s="4"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="2" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B60" s="3" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="B60" s="3" t="s">
+      <x:c r="C60" s="4" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="C60" s="4" t="s">
-        <x:v>150</x:v>
       </x:c>
       <x:c r="D60" s="4"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="2" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B61" s="3" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="B61" s="3" t="s">
+      <x:c r="C61" s="4" t="s">
         <x:v>152</x:v>
-      </x:c>
-      <x:c r="C61" s="4" t="s">
-        <x:v>153</x:v>
       </x:c>
       <x:c r="D61" s="4"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="B62" s="3" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="B62" s="3" t="s">
+      <x:c r="C62" s="4" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="C62" s="4" t="s">
+      <x:c r="D62" s="4" t="s">
         <x:v>156</x:v>
-      </x:c>
-      <x:c r="D62" s="4" t="s">
-        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B63" s="6" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="B63" s="6" t="s">
+      <x:c r="C63" s="7" t="s">
         <x:v>159</x:v>
-      </x:c>
-      <x:c r="C63" s="7" t="s">
-        <x:v>160</x:v>
       </x:c>
       <x:c r="D63" s="7"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="12" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="B64" s="13" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="B64" s="13" t="s">
+      <x:c r="C64" s="14" t="s">
         <x:v>162</x:v>
-      </x:c>
-      <x:c r="C64" s="14" t="s">
-        <x:v>163</x:v>
       </x:c>
       <x:c r="D64" s="14"/>
     </x:row>
     <x:row r="65" ht="28.5">
       <x:c r="A65" s="15" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="B65" s="16" t="s">
+      <x:c r="C65" s="4" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="C65" s="4" t="s">
-        <x:v>166</x:v>
-      </x:c>
       <x:c r="D65" s="4" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="15" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="B66" s="16" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="B66" s="16" t="s">
+      <x:c r="C66" s="4" t="s">
         <x:v>168</x:v>
-      </x:c>
-      <x:c r="C66" s="4" t="s">
-        <x:v>169</x:v>
       </x:c>
       <x:c r="D66" s="4"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="15" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="B67" s="16" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="B67" s="16" t="s">
+      <x:c r="C67" s="4" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="C67" s="4" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="D67" s="4"/>
     </x:row>
     <x:row r="68" ht="28.5">
       <x:c r="A68" s="15" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="B68" s="16" t="s">
         <x:v>173</x:v>
       </x:c>
-      <x:c r="B68" s="16" t="s">
-        <x:v>174</x:v>
-      </x:c>
       <x:c r="C68" s="4" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D68" s="4"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="15" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="B69" s="16" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="B69" s="16" t="s">
+      <x:c r="C69" s="4" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="C69" s="4" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="D69" s="4"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="15" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B70" s="16" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="B70" s="16" t="s">
+      <x:c r="C70" s="4" t="s">
         <x:v>179</x:v>
-      </x:c>
-      <x:c r="C70" s="4" t="s">
-        <x:v>180</x:v>
       </x:c>
       <x:c r="D70" s="4"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="15" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B71" s="16" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="B71" s="16" t="s">
+      <x:c r="C71" s="4" t="s">
         <x:v>182</x:v>
-      </x:c>
-      <x:c r="C71" s="4" t="s">
-        <x:v>183</x:v>
       </x:c>
       <x:c r="D71" s="4"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="15" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="B72" s="16" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="B72" s="16" t="s">
+      <x:c r="C72" s="4" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="C72" s="4" t="s">
+      <x:c r="D72" s="4" t="s">
         <x:v>186</x:v>
-      </x:c>
-      <x:c r="D72" s="4" t="s">
-        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="15" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B73" s="16" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="B73" s="16" t="s">
+      <x:c r="C73" s="4" t="s">
         <x:v>189</x:v>
-      </x:c>
-      <x:c r="C73" s="4" t="s">
-        <x:v>190</x:v>
       </x:c>
       <x:c r="D73" s="4"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="15" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="B74" s="16" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="B74" s="16" t="s">
-        <x:v>192</x:v>
-      </x:c>
       <x:c r="C74" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D74" s="4"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="15" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B75" s="16" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="B75" s="16" t="s">
-        <x:v>194</x:v>
-      </x:c>
       <x:c r="C75" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D75" s="4"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="15" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="B76" s="16" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="B76" s="16" t="s">
+      <x:c r="C76" s="4" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="C76" s="4" t="s">
-        <x:v>197</x:v>
       </x:c>
       <x:c r="D76" s="4"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="15" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B77" s="16" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="B77" s="16" t="s">
+      <x:c r="C77" s="4" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="C77" s="4" t="s">
-        <x:v>200</x:v>
       </x:c>
       <x:c r="D77" s="4"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="15" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B78" s="16" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="B78" s="16" t="s">
+      <x:c r="C78" s="4" t="s">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="C78" s="4" t="s">
-        <x:v>203</x:v>
       </x:c>
       <x:c r="D78" s="4"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="15" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B79" s="16" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="B79" s="16" t="s">
+      <x:c r="C79" s="4" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="C79" s="4" t="s">
+      <x:c r="D79" s="4" t="s">
         <x:v>206</x:v>
-      </x:c>
-      <x:c r="D79" s="4" t="s">
-        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="17" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B80" s="18" t="s">
         <x:v>208</x:v>
       </x:c>
-      <x:c r="B80" s="18" t="s">
-        <x:v>209</x:v>
-      </x:c>
       <x:c r="C80" s="7" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D80" s="7"/>
     </x:row>
     <x:row r="81" ht="14.25" customHeight="1">
       <x:c r="A81" s="19" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="B81" s="21" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="B81" s="21" t="s">
+      <x:c r="C81" s="23" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="C81" s="23" t="s">
+      <x:c r="D81" s="23" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="D81" s="23" t="s">
-        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="14.25" customHeight="1">
       <x:c r="A82" s="19" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B82" s="21" t="s">
         <x:v>214</x:v>
       </x:c>
-      <x:c r="B82" s="21" t="s">
+      <x:c r="C82" s="23" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="C82" s="23" t="s">
-        <x:v>216</x:v>
-      </x:c>
       <x:c r="D82" s="23" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="14.25" customHeight="1">
       <x:c r="A83" s="19" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="B83" s="21" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="B83" s="21" t="s">
+      <x:c r="C83" s="23" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="C83" s="23" t="s">
-        <x:v>219</x:v>
-      </x:c>
       <x:c r="D83" s="23" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="14.25" customHeight="1">
       <x:c r="A84" s="19" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="B84" s="21" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="B84" s="21" t="s">
+      <x:c r="C84" s="23" t="s">
         <x:v>221</x:v>
-      </x:c>
-      <x:c r="C84" s="23" t="s">
-        <x:v>222</x:v>
       </x:c>
       <x:c r="D84" s="23"/>
     </x:row>
     <x:row r="85" ht="14.25" customHeight="1">
       <x:c r="A85" s="19" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="B85" s="21" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="B85" s="21" t="s">
+      <x:c r="C85" s="23" t="s">
         <x:v>224</x:v>
-      </x:c>
-      <x:c r="C85" s="23" t="s">
-        <x:v>225</x:v>
       </x:c>
       <x:c r="D85" s="23"/>
     </x:row>
     <x:row r="86" ht="14.25" customHeight="1">
       <x:c r="A86" s="19" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="B86" s="21" t="s">
         <x:v>226</x:v>
       </x:c>
-      <x:c r="B86" s="21" t="s">
+      <x:c r="C86" s="23" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="C86" s="23" t="s">
-        <x:v>228</x:v>
       </x:c>
       <x:c r="D86" s="23"/>
     </x:row>
     <x:row r="87" ht="14.25" customHeight="1">
       <x:c r="A87" s="19" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="B87" s="21" t="s">
         <x:v>229</x:v>
       </x:c>
-      <x:c r="B87" s="21" t="s">
-        <x:v>230</x:v>
-      </x:c>
       <x:c r="C87" s="23" t="s">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="D87" s="23" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="26.450000762939453" customHeight="1">
       <x:c r="A88" s="19" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="B88" s="21" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="B88" s="21" t="s">
+      <x:c r="C88" s="23" t="s">
         <x:v>232</x:v>
       </x:c>
-      <x:c r="C88" s="23" t="s">
+      <x:c r="D88" s="23" t="s">
         <x:v>233</x:v>
-      </x:c>
-      <x:c r="D88" s="23" t="s">
-        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="14.25" customHeight="1">
       <x:c r="A89" s="19" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="B89" s="21" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="B89" s="21" t="s">
+      <x:c r="C89" s="23" t="s">
         <x:v>236</x:v>
-      </x:c>
-      <x:c r="C89" s="23" t="s">
-        <x:v>237</x:v>
       </x:c>
       <x:c r="D89" s="23"/>
     </x:row>
     <x:row r="90" ht="14.25" customHeight="1">
       <x:c r="A90" s="19" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B90" s="21" t="s">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="B90" s="21" t="s">
-        <x:v>239</x:v>
-      </x:c>
       <x:c r="C90" s="23" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="D90" s="23"/>
     </x:row>
     <x:row r="91" ht="14.25" customHeight="1">
       <x:c r="A91" s="19" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="B91" s="21" t="s">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="B91" s="21" t="s">
-        <x:v>241</x:v>
-      </x:c>
       <x:c r="C91" s="23" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="D91" s="23"/>
     </x:row>
     <x:row r="92" ht="14.25" customHeight="1">
       <x:c r="A92" s="19" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="B92" s="21" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="B92" s="21" t="s">
-        <x:v>243</x:v>
-      </x:c>
       <x:c r="C92" s="23" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="D92" s="23"/>
     </x:row>
     <x:row r="93" ht="14.25" customHeight="1">
       <x:c r="A93" s="20" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="B93" s="22" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="B93" s="22" t="s">
+      <x:c r="C93" s="24" t="s">
         <x:v>245</x:v>
-      </x:c>
-      <x:c r="C93" s="24" t="s">
-        <x:v>246</x:v>
       </x:c>
       <x:c r="D93" s="24"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="26" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="B94" s="29" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="B94" s="29" t="s">
+      <x:c r="C94" s="32" t="s">
         <x:v>248</x:v>
-      </x:c>
-      <x:c r="C94" s="32" t="s">
-        <x:v>249</x:v>
       </x:c>
       <x:c r="D94" s="32"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="27" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="B95" s="30" t="s">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="B95" s="30" t="s">
+      <x:c r="C95" s="33" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="C95" s="33" t="s">
+      <x:c r="D95" s="33" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="D95" s="33" t="s">
-        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="27" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="B96" s="30" t="s">
         <x:v>254</x:v>
       </x:c>
-      <x:c r="B96" s="30" t="s">
+      <x:c r="C96" s="34" t="s">
         <x:v>255</x:v>
-      </x:c>
-      <x:c r="C96" s="34" t="s">
-        <x:v>256</x:v>
       </x:c>
       <x:c r="D96" s="34"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="27" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="B97" s="30" t="s">
         <x:v>257</x:v>
       </x:c>
-      <x:c r="B97" s="30" t="s">
+      <x:c r="C97" s="33" t="s">
         <x:v>258</x:v>
-      </x:c>
-      <x:c r="C97" s="33" t="s">
-        <x:v>259</x:v>
       </x:c>
       <x:c r="D97" s="33"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="27" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B98" s="30" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="B98" s="30" t="s">
+      <x:c r="C98" s="34" t="s">
         <x:v>261</x:v>
-      </x:c>
-      <x:c r="C98" s="34" t="s">
-        <x:v>262</x:v>
       </x:c>
       <x:c r="D98" s="34"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="27" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="B99" s="30" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="B99" s="30" t="s">
+      <x:c r="C99" s="33" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="C99" s="33" t="s">
-        <x:v>265</x:v>
       </x:c>
       <x:c r="D99" s="33"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="27" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="B100" s="30" t="s">
         <x:v>266</x:v>
       </x:c>
-      <x:c r="B100" s="30" t="s">
+      <x:c r="C100" s="34" t="s">
         <x:v>267</x:v>
-      </x:c>
-      <x:c r="C100" s="34" t="s">
-        <x:v>268</x:v>
       </x:c>
       <x:c r="D100" s="34"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="27" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="B101" s="30" t="s">
         <x:v>269</x:v>
       </x:c>
-      <x:c r="B101" s="30" t="s">
+      <x:c r="C101" s="33" t="s">
         <x:v>270</x:v>
-      </x:c>
-      <x:c r="C101" s="33" t="s">
-        <x:v>271</x:v>
       </x:c>
       <x:c r="D101" s="33"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="27" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="B102" s="30" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="B102" s="30" t="s">
+      <x:c r="C102" s="34" t="s">
         <x:v>273</x:v>
-      </x:c>
-      <x:c r="C102" s="34" t="s">
-        <x:v>274</x:v>
       </x:c>
       <x:c r="D102" s="34"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="27" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="B103" s="30" t="s">
         <x:v>275</x:v>
       </x:c>
-      <x:c r="B103" s="30" t="s">
+      <x:c r="C103" s="33" t="s">
         <x:v>276</x:v>
-      </x:c>
-      <x:c r="C103" s="33" t="s">
-        <x:v>277</x:v>
       </x:c>
       <x:c r="D103" s="33"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="27" t="s">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="B104" s="30" t="s">
         <x:v>278</x:v>
       </x:c>
-      <x:c r="B104" s="30" t="s">
+      <x:c r="C104" s="34" t="s">
         <x:v>279</x:v>
-      </x:c>
-      <x:c r="C104" s="34" t="s">
-        <x:v>280</x:v>
       </x:c>
       <x:c r="D104" s="34"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="27" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="B105" s="30" t="s">
         <x:v>281</x:v>
       </x:c>
-      <x:c r="B105" s="30" t="s">
+      <x:c r="C105" s="33" t="s">
         <x:v>282</x:v>
-      </x:c>
-      <x:c r="C105" s="33" t="s">
-        <x:v>283</x:v>
       </x:c>
       <x:c r="D105" s="33"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="27" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B106" s="30" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="B106" s="30" t="s">
-        <x:v>285</x:v>
-      </x:c>
       <x:c r="C106" s="34" t="s">
-        <x:v>283</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="D106" s="34"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="27" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="B107" s="30" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="B107" s="30" t="s">
+      <x:c r="C107" s="33" t="s">
         <x:v>287</x:v>
-      </x:c>
-      <x:c r="C107" s="33" t="s">
-        <x:v>288</x:v>
       </x:c>
       <x:c r="D107" s="33"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="27" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="B108" s="30" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="B108" s="30" t="s">
+      <x:c r="C108" s="34" t="s">
         <x:v>290</x:v>
-      </x:c>
-      <x:c r="C108" s="34" t="s">
-        <x:v>291</x:v>
       </x:c>
       <x:c r="D108" s="34"/>
     </x:row>
     <x:row r="109" ht="28.5">
       <x:c r="A109" s="27" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B109" s="30" t="s">
         <x:v>292</x:v>
       </x:c>
-      <x:c r="B109" s="30" t="s">
+      <x:c r="C109" s="33" t="s">
         <x:v>293</x:v>
-      </x:c>
-      <x:c r="C109" s="33" t="s">
-        <x:v>294</x:v>
       </x:c>
       <x:c r="D109" s="33"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="27" t="s">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="B110" s="30" t="s">
         <x:v>295</x:v>
       </x:c>
-      <x:c r="B110" s="30" t="s">
+      <x:c r="C110" s="34" t="s">
         <x:v>296</x:v>
-      </x:c>
-      <x:c r="C110" s="34" t="s">
-        <x:v>297</x:v>
       </x:c>
       <x:c r="D110" s="34"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="27" t="s">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="B111" s="30" t="s">
         <x:v>298</x:v>
       </x:c>
-      <x:c r="B111" s="30" t="s">
+      <x:c r="C111" s="33" t="s">
         <x:v>299</x:v>
-      </x:c>
-      <x:c r="C111" s="33" t="s">
-        <x:v>300</x:v>
       </x:c>
       <x:c r="D111" s="33"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="28" t="s">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="B112" s="31" t="s">
         <x:v>301</x:v>
       </x:c>
-      <x:c r="B112" s="31" t="s">
+      <x:c r="C112" s="35" t="s">
         <x:v>302</x:v>
-      </x:c>
-      <x:c r="C112" s="35" t="s">
-        <x:v>303</x:v>
       </x:c>
       <x:c r="D112" s="35"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="s">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="B113" t="s">
         <x:v>304</x:v>
       </x:c>
-      <x:c r="B113" t="s">
+      <x:c r="C113" t="s">
         <x:v>305</x:v>
-      </x:c>
-      <x:c r="C113" t="s">
-        <x:v>306</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="B114" t="s">
         <x:v>307</x:v>
       </x:c>
-      <x:c r="B114" t="s">
-        <x:v>308</x:v>
-      </x:c>
       <x:c r="C114" t="s">
-        <x:v>306</x:v>
+        <x:v>305</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="B115" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="B115" t="s">
+      <x:c r="C115" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="C115" t="s">
+      <x:c r="D115" t="s">
         <x:v>311</x:v>
-      </x:c>
-      <x:c r="D115" t="s">
-        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="B116" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="B116" t="s">
+      <x:c r="C116" t="s">
         <x:v>314</x:v>
       </x:c>
-      <x:c r="C116" t="s">
+      <x:c r="D116" t="s">
         <x:v>315</x:v>
-      </x:c>
-      <x:c r="D116" t="s">
-        <x:v>316</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="B117" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="B117" t="s">
+      <x:c r="C117" t="s">
         <x:v>318</x:v>
-      </x:c>
-      <x:c r="C117" t="s">
-        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="36" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B118" s="39" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="B118" s="39" t="s">
+      <x:c r="C118" s="25" t="s">
         <x:v>321</x:v>
       </x:c>
-      <x:c r="C118" s="25" t="s">
+      <x:c r="D118" s="25" t="s">
         <x:v>322</x:v>
-      </x:c>
-      <x:c r="D118" s="25" t="s">
-        <x:v>323</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="37" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="B119" s="40" t="s">
         <x:v>324</x:v>
       </x:c>
-      <x:c r="B119" s="40" t="s">
+      <x:c r="C119" s="11" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="D119" s="11" t="s">
         <x:v>325</x:v>
-      </x:c>
-      <x:c r="C119" s="11" t="s">
-        <x:v>322</x:v>
-      </x:c>
-      <x:c r="D119" s="11" t="s">
-        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="37" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="B120" s="40" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="B120" s="40" t="s">
+      <x:c r="C120" s="11" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="C120" s="11" t="s">
+      <x:c r="D120" s="11" t="s">
         <x:v>329</x:v>
-      </x:c>
-      <x:c r="D120" s="11" t="s">
-        <x:v>330</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="28.5">
       <x:c r="A121" s="37" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="B121" s="40" t="s">
         <x:v>331</x:v>
       </x:c>
-      <x:c r="B121" s="40" t="s">
+      <x:c r="C121" s="11" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="C121" s="11" t="s">
+      <x:c r="D121" s="11" t="s">
         <x:v>333</x:v>
-      </x:c>
-      <x:c r="D121" s="11" t="s">
-        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="28.5">
       <x:c r="A122" s="37" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="B122" s="40" t="s">
         <x:v>335</x:v>
       </x:c>
-      <x:c r="B122" s="40" t="s">
+      <x:c r="C122" s="11" t="s">
         <x:v>336</x:v>
       </x:c>
-      <x:c r="C122" s="11" t="s">
+      <x:c r="D122" s="11" t="s">
         <x:v>337</x:v>
-      </x:c>
-      <x:c r="D122" s="11" t="s">
-        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="37" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="B123" s="40" t="s">
         <x:v>339</x:v>
       </x:c>
-      <x:c r="B123" s="40" t="s">
+      <x:c r="C123" s="11" t="s">
         <x:v>340</x:v>
-      </x:c>
-      <x:c r="C123" s="11" t="s">
-        <x:v>341</x:v>
       </x:c>
       <x:c r="D123" s="11"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="37" t="s">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B124" s="40" t="s">
         <x:v>342</x:v>
       </x:c>
-      <x:c r="B124" s="40" t="s">
+      <x:c r="C124" s="11" t="s">
         <x:v>343</x:v>
-      </x:c>
-      <x:c r="C124" s="11" t="s">
-        <x:v>344</x:v>
       </x:c>
       <x:c r="D124" s="11"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="37" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B125" s="40" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="B125" s="40" t="s">
+      <x:c r="C125" s="11" t="s">
         <x:v>346</x:v>
-      </x:c>
-      <x:c r="C125" s="11" t="s">
-        <x:v>347</x:v>
       </x:c>
       <x:c r="D125" s="11"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="37" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B126" s="40" t="s">
         <x:v>348</x:v>
       </x:c>
-      <x:c r="B126" s="40" t="s">
+      <x:c r="C126" s="11" t="s">
         <x:v>349</x:v>
-      </x:c>
-      <x:c r="C126" s="11" t="s">
-        <x:v>350</x:v>
       </x:c>
       <x:c r="D126" s="11"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="37" t="s">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="B127" s="40" t="s">
         <x:v>351</x:v>
       </x:c>
-      <x:c r="B127" s="40" t="s">
-        <x:v>352</x:v>
-      </x:c>
       <x:c r="C127" s="11" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D127" s="11"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="37" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="B128" s="40" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="B128" s="40" t="s">
-        <x:v>354</x:v>
-      </x:c>
       <x:c r="C128" s="11" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D128" s="11"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="37" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B129" s="40" t="s">
         <x:v>355</x:v>
       </x:c>
-      <x:c r="B129" s="40" t="s">
-        <x:v>356</x:v>
-      </x:c>
       <x:c r="C129" s="11" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D129" s="11"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="37" t="s">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="B130" s="40" t="s">
         <x:v>357</x:v>
       </x:c>
-      <x:c r="B130" s="40" t="s">
-        <x:v>358</x:v>
-      </x:c>
       <x:c r="C130" s="11" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="D130" s="11"/>
     </x:row>
     <x:row r="131" ht="28.5">
       <x:c r="A131" s="37" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B131" s="40" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="B131" s="40" t="s">
+      <x:c r="C131" s="11" t="s">
         <x:v>360</x:v>
-      </x:c>
-      <x:c r="C131" s="11" t="s">
-        <x:v>361</x:v>
       </x:c>
       <x:c r="D131" s="11"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="37" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="B132" s="40" t="s">
         <x:v>362</x:v>
       </x:c>
-      <x:c r="B132" s="40" t="s">
+      <x:c r="C132" s="11" t="s">
         <x:v>363</x:v>
-      </x:c>
-      <x:c r="C132" s="11" t="s">
-        <x:v>364</x:v>
       </x:c>
       <x:c r="D132" s="11"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="37" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="B133" s="40" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="B133" s="40" t="s">
+      <x:c r="C133" s="11" t="s">
         <x:v>366</x:v>
-      </x:c>
-      <x:c r="C133" s="11" t="s">
-        <x:v>367</x:v>
       </x:c>
       <x:c r="D133" s="11"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="37" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="B134" s="40" t="s">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="B134" s="40" t="s">
+      <x:c r="C134" s="11" t="s">
         <x:v>369</x:v>
-      </x:c>
-      <x:c r="C134" s="11" t="s">
-        <x:v>370</x:v>
       </x:c>
       <x:c r="D134" s="11"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="38" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="B135" s="41" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="B135" s="41" t="s">
-        <x:v>372</x:v>
-      </x:c>
       <x:c r="C135" s="14" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="D135" s="14"/>
     </x:row>
     <x:row r="136" ht="28.5">
       <x:c r="A136" s="42" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="B136" s="44" t="s">
         <x:v>373</x:v>
       </x:c>
-      <x:c r="B136" s="44" t="s">
+      <x:c r="C136" s="14" t="s">
         <x:v>374</x:v>
       </x:c>
-      <x:c r="C136" s="14" t="s">
+      <x:c r="D136" s="14" t="s">
         <x:v>375</x:v>
-      </x:c>
-      <x:c r="D136" s="14" t="s">
-        <x:v>376</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="43" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="B137" s="45" t="s">
         <x:v>377</x:v>
       </x:c>
-      <x:c r="B137" s="45" t="s">
+      <x:c r="C137" s="4" t="s">
         <x:v>378</x:v>
-      </x:c>
-      <x:c r="C137" s="4" t="s">
-        <x:v>379</x:v>
       </x:c>
       <x:c r="D137" s="4"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="43" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="B138" s="45" t="s">
         <x:v>380</x:v>
       </x:c>
-      <x:c r="B138" s="45" t="s">
+      <x:c r="C138" s="4" t="s">
         <x:v>381</x:v>
-      </x:c>
-      <x:c r="C138" s="4" t="s">
-        <x:v>382</x:v>
       </x:c>
       <x:c r="D138" s="4"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="43" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="B139" s="45" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="B139" s="45" t="s">
-        <x:v>384</x:v>
-      </x:c>
       <x:c r="C139" s="4" t="s">
-        <x:v>382</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="D139" s="4"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="43" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="B140" s="45" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="B140" s="45" t="s">
-        <x:v>386</x:v>
-      </x:c>
       <x:c r="C140" s="4" t="s">
-        <x:v>382</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="D140" s="4"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="43" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="B141" s="45" t="s">
         <x:v>387</x:v>
       </x:c>
-      <x:c r="B141" s="45" t="s">
+      <x:c r="C141" s="4" t="s">
         <x:v>388</x:v>
-      </x:c>
-      <x:c r="C141" s="4" t="s">
-        <x:v>389</x:v>
       </x:c>
       <x:c r="D141" s="4"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="43" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="B142" s="45" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="B142" s="45" t="s">
+      <x:c r="C142" s="4" t="s">
         <x:v>391</x:v>
-      </x:c>
-      <x:c r="C142" s="4" t="s">
-        <x:v>392</x:v>
       </x:c>
       <x:c r="D142" s="4"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="43" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="B143" s="45" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="B143" s="45" t="s">
-        <x:v>394</x:v>
-      </x:c>
       <x:c r="C143" s="4" t="s">
-        <x:v>392</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="D143" s="4"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="43" t="s">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="B144" s="45" t="s">
         <x:v>395</x:v>
       </x:c>
-      <x:c r="B144" s="45" t="s">
+      <x:c r="C144" s="4" t="s">
         <x:v>396</x:v>
-      </x:c>
-      <x:c r="C144" s="4" t="s">
-        <x:v>397</x:v>
       </x:c>
       <x:c r="D144" s="4"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="43" t="s">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="B145" s="45" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="B145" s="45" t="s">
+      <x:c r="C145" s="4" t="s">
         <x:v>399</x:v>
-      </x:c>
-      <x:c r="C145" s="4" t="s">
-        <x:v>400</x:v>
       </x:c>
       <x:c r="D145" s="4"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="43" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="B146" s="45" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="B146" s="45" t="s">
+      <x:c r="C146" s="4" t="s">
         <x:v>402</x:v>
-      </x:c>
-      <x:c r="C146" s="4" t="s">
-        <x:v>403</x:v>
       </x:c>
       <x:c r="D146" s="4"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="43" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="B147" s="45" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="B147" s="45" t="s">
+      <x:c r="C147" s="4" t="s">
         <x:v>405</x:v>
-      </x:c>
-      <x:c r="C147" s="4" t="s">
-        <x:v>406</x:v>
       </x:c>
       <x:c r="D147" s="4"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="43" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="B148" s="45" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="B148" s="45" t="s">
+      <x:c r="C148" s="4" t="s">
         <x:v>408</x:v>
-      </x:c>
-      <x:c r="C148" s="4" t="s">
-        <x:v>409</x:v>
       </x:c>
       <x:c r="D148" s="4"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="43" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="B149" s="45" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="B149" s="45" t="s">
+      <x:c r="C149" s="4" t="s">
         <x:v>411</x:v>
-      </x:c>
-      <x:c r="C149" s="4" t="s">
-        <x:v>412</x:v>
       </x:c>
       <x:c r="D149" s="4"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="43" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="B150" s="45" t="s">
         <x:v>413</x:v>
       </x:c>
-      <x:c r="B150" s="45" t="s">
+      <x:c r="C150" s="4" t="s">
         <x:v>414</x:v>
-      </x:c>
-      <x:c r="C150" s="4" t="s">
-        <x:v>415</x:v>
       </x:c>
       <x:c r="D150" s="4"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="43" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="B151" s="45" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="C151" s="4" t="s">
         <x:v>416</x:v>
-      </x:c>
-      <x:c r="B151" s="45" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="C151" s="4" t="s">
-        <x:v>417</x:v>
       </x:c>
       <x:c r="D151" s="4"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="43" t="s">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="B152" s="45" t="s">
         <x:v>418</x:v>
       </x:c>
-      <x:c r="B152" s="45" t="s">
+      <x:c r="C152" s="4" t="s">
         <x:v>419</x:v>
-      </x:c>
-      <x:c r="C152" s="4" t="s">
-        <x:v>420</x:v>
       </x:c>
       <x:c r="D152" s="4"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" t="s">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="B153" t="s">
         <x:v>421</x:v>
       </x:c>
-      <x:c r="B153" t="s">
+      <x:c r="C153" t="s">
         <x:v>422</x:v>
-      </x:c>
-      <x:c r="C153" t="s">
-        <x:v>423</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" t="s">
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="B154" t="s">
         <x:v>424</x:v>
       </x:c>
-      <x:c r="B154" t="s">
-        <x:v>425</x:v>
-      </x:c>
       <x:c r="C154" t="s">
-        <x:v>423</x:v>
+        <x:v>422</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" t="s">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="B155" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="B155" t="s">
-        <x:v>427</x:v>
-      </x:c>
       <x:c r="C155" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
       <x:c r="A156" t="s">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="B156" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="B156" t="s">
-        <x:v>429</x:v>
-      </x:c>
       <x:c r="C156" t="s">
-        <x:v>341</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
       <x:c r="A157" t="s">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="B157" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="B157" t="s">
-        <x:v>431</x:v>
-      </x:c>
       <x:c r="C157" t="s">
-        <x:v>341</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
       <x:c r="A158" t="s">
+        <x:v>431</x:v>
+      </x:c>
+      <x:c r="B158" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="B158" t="s">
+      <x:c r="C158" t="s">
         <x:v>433</x:v>
-      </x:c>
-      <x:c r="C158" t="s">
-        <x:v>434</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="20.100000381469727" customHeight="1">
       <x:c r="A159" s="46" t="s">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="B159" s="47" t="s">
         <x:v>435</x:v>
       </x:c>
-      <x:c r="B159" s="47" t="s">
+      <x:c r="C159" s="48" t="s">
         <x:v>436</x:v>
-      </x:c>
-      <x:c r="C159" s="48" t="s">
-        <x:v>437</x:v>
       </x:c>
       <x:c r="D159" s="4"/>
     </x:row>
     <x:row r="160" ht="20.100000381469727" customHeight="1">
       <x:c r="A160" s="46" t="s">
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="B160" s="47" t="s">
         <x:v>438</x:v>
       </x:c>
-      <x:c r="B160" s="47" t="s">
+      <x:c r="C160" s="48" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="C160" s="48" t="s">
+      <x:c r="D160" s="4" t="s">
         <x:v>440</x:v>
-      </x:c>
-      <x:c r="D160" s="4" t="s">
-        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="161">
       <x:c r="A161" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="B161" t="s">
         <x:v>442</x:v>
       </x:c>
-      <x:c r="B161" t="s">
-        <x:v>443</x:v>
-      </x:c>
       <x:c r="C161" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
       <x:c r="A162" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="B162" t="s">
         <x:v>444</x:v>
       </x:c>
-      <x:c r="B162" t="s">
-        <x:v>445</x:v>
-      </x:c>
       <x:c r="C162" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="163">
       <x:c r="A163" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="B163" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="B163" t="s">
+      <x:c r="C163" t="s">
         <x:v>447</x:v>
-      </x:c>
-      <x:c r="C163" t="s">
-        <x:v>448</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
       <x:c r="A164" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="B164" t="s">
         <x:v>449</x:v>
       </x:c>
-      <x:c r="B164" t="s">
-        <x:v>450</x:v>
-      </x:c>
       <x:c r="C164" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
       <x:c r="A165" t="s">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="B165" t="s">
         <x:v>451</x:v>
       </x:c>
-      <x:c r="B165" t="s">
-        <x:v>452</x:v>
-      </x:c>
       <x:c r="C165" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="B166" t="s">
         <x:v>453</x:v>
       </x:c>
-      <x:c r="B166" t="s">
-        <x:v>454</x:v>
-      </x:c>
       <x:c r="C166" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
       <x:c r="A167" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="B167" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="B167" t="s">
-        <x:v>456</x:v>
-      </x:c>
       <x:c r="C167" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="B168" t="s">
         <x:v>457</x:v>
       </x:c>
-      <x:c r="B168" t="s">
-        <x:v>458</x:v>
-      </x:c>
       <x:c r="C168" t="s">
-        <x:v>448</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
       <x:c r="A169" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="B169" t="s">
         <x:v>459</x:v>
       </x:c>
-      <x:c r="B169" t="s">
+      <x:c r="C169" t="s">
         <x:v>460</x:v>
-      </x:c>
-      <x:c r="C169" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
       <x:c r="A170" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="B170" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="B170" t="s">
-        <x:v>463</x:v>
       </x:c>
       <x:c r="C170" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="D170" t="s">
-        <x:v>464</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
       <x:c r="A171" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="B171" t="s">
         <x:v>465</x:v>
-      </x:c>
-      <x:c r="B171" t="s">
-        <x:v>466</x:v>
       </x:c>
       <x:c r="C171" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="D171" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
       <x:c r="A172" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B172" t="s">
         <x:v>21</x:v>
@@ -4134,119 +4131,119 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="D172" t="s">
-        <x:v>464</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
       <x:c r="A173" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="B173" t="s">
         <x:v>469</x:v>
-      </x:c>
-      <x:c r="B173" t="s">
-        <x:v>470</x:v>
       </x:c>
       <x:c r="C173" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="D173" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
       <x:c r="A174" t="s">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="B174" t="s">
         <x:v>472</x:v>
-      </x:c>
-      <x:c r="B174" t="s">
-        <x:v>473</x:v>
       </x:c>
       <x:c r="C174" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="D174" t="s">
-        <x:v>464</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
       <x:c r="A175" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="B175" t="s">
         <x:v>474</x:v>
       </x:c>
-      <x:c r="B175" t="s">
+      <x:c r="C175" t="s">
         <x:v>475</x:v>
       </x:c>
-      <x:c r="C175" t="s">
+      <x:c r="D175" t="s">
         <x:v>476</x:v>
-      </x:c>
-      <x:c r="D175" t="s">
-        <x:v>477</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
       <x:c r="A176" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="B176" t="s">
         <x:v>478</x:v>
       </x:c>
-      <x:c r="B176" t="s">
+      <x:c r="C176" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="D176" t="s">
         <x:v>479</x:v>
-      </x:c>
-      <x:c r="C176" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="D176" t="s">
-        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
       <x:c r="A177" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="B177" t="s">
         <x:v>481</x:v>
       </x:c>
-      <x:c r="B177" t="s">
-        <x:v>482</x:v>
-      </x:c>
       <x:c r="C177" t="s">
-        <x:v>476</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="D177" t="s">
-        <x:v>480</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
       <x:c r="A178" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="B178" t="s">
         <x:v>483</x:v>
       </x:c>
-      <x:c r="B178" t="s">
-        <x:v>484</x:v>
-      </x:c>
       <x:c r="C178" t="s">
-        <x:v>476</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="D178" t="s">
-        <x:v>480</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
       <x:c r="A179" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="B179" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="B179" t="s">
+      <x:c r="C179" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="D179" t="s">
         <x:v>486</x:v>
-      </x:c>
-      <x:c r="C179" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="D179" t="s">
-        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
       <x:c r="A180" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="B180" t="s">
         <x:v>488</x:v>
       </x:c>
-      <x:c r="B180" t="s">
+      <x:c r="C180" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="D180" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="C180" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="D180" t="s">
-        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -4270,7 +4267,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8ff5cd7e1854c16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd30d58cb154a3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,56 +4282,56 @@
   <x:sheetData>
     <x:row r="1" ht="32.099998474121094" customHeight="1">
       <x:c r="A1" s="51" t="s">
-        <x:v>491</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B1" s="51"/>
     </x:row>
     <x:row r="3" ht="15">
       <x:c r="A3" s="8" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="s">
         <x:v>492</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="s">
-        <x:v>493</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
       <x:c r="A4" s="8" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="s">
         <x:v>494</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="s">
-        <x:v>495</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15">
       <x:c r="A5" s="8" t="s">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="s">
         <x:v>496</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="s">
-        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15">
       <x:c r="A6" s="8" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="s">
         <x:v>498</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="s">
-        <x:v>499</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15">
       <x:c r="A7" s="8" t="s">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="s">
         <x:v>500</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="s">
-        <x:v>501</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="10" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="s">
         <x:v>502</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="s">
-        <x:v>503</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>